<commit_message>
keyrðu út frá nýju input
</commit_message>
<xml_diff>
--- a/Data/04_26_schedule_results.xlsx
+++ b/Data/04_26_schedule_results.xlsx
@@ -586,15 +586,15 @@
       </c>
       <c r="G3" t="inlineStr"/>
       <c r="H3" t="n">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>Ömmi</t>
+          <t xml:space="preserve">Þórey </t>
         </is>
       </c>
       <c r="J3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K3" t="n">
         <v>0</v>
@@ -606,7 +606,7 @@
         <v>100</v>
       </c>
       <c r="N3" t="n">
-        <v>490</v>
+        <v>520</v>
       </c>
     </row>
     <row r="4">
@@ -638,11 +638,11 @@
       </c>
       <c r="G4" t="inlineStr"/>
       <c r="H4" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Anna Soffía </t>
+          <t xml:space="preserve">Elísabet </t>
         </is>
       </c>
       <c r="J4" t="n">
@@ -658,7 +658,7 @@
         <v>70</v>
       </c>
       <c r="N4" t="n">
-        <v>520</v>
+        <v>610</v>
       </c>
     </row>
     <row r="5">
@@ -690,18 +690,18 @@
       </c>
       <c r="G5" t="inlineStr"/>
       <c r="H5" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Elísabet </t>
+          <t>Gréta</t>
         </is>
       </c>
       <c r="J5" t="n">
         <v>2</v>
       </c>
       <c r="K5" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="L5" t="n">
         <v>3.5</v>
@@ -710,7 +710,7 @@
         <v>70</v>
       </c>
       <c r="N5" t="n">
-        <v>610</v>
+        <v>400</v>
       </c>
     </row>
     <row r="6">
@@ -742,18 +742,18 @@
       </c>
       <c r="G6" t="inlineStr"/>
       <c r="H6" t="n">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Elmar </t>
+          <t xml:space="preserve">Guðný  </t>
         </is>
       </c>
       <c r="J6" t="n">
         <v>2</v>
       </c>
       <c r="K6" t="n">
-        <v>12</v>
+        <v>3</v>
       </c>
       <c r="L6" t="n">
         <v>3.5</v>
@@ -762,7 +762,7 @@
         <v>70</v>
       </c>
       <c r="N6" t="n">
-        <v>612.3</v>
+        <v>400</v>
       </c>
     </row>
     <row r="7">
@@ -794,18 +794,18 @@
       </c>
       <c r="G7" t="inlineStr"/>
       <c r="H7" t="n">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>Gréta</t>
+          <t>Hrafnkell</t>
         </is>
       </c>
       <c r="J7" t="n">
         <v>2</v>
       </c>
       <c r="K7" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="L7" t="n">
         <v>3.5</v>
@@ -814,7 +814,7 @@
         <v>70</v>
       </c>
       <c r="N7" t="n">
-        <v>400</v>
+        <v>610</v>
       </c>
     </row>
     <row r="8">
@@ -846,18 +846,18 @@
       </c>
       <c r="G8" t="inlineStr"/>
       <c r="H8" t="n">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Guðný  </t>
+          <t xml:space="preserve">Jórunn  </t>
         </is>
       </c>
       <c r="J8" t="n">
         <v>2</v>
       </c>
       <c r="K8" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="L8" t="n">
         <v>3.5</v>
@@ -866,7 +866,7 @@
         <v>70</v>
       </c>
       <c r="N8" t="n">
-        <v>400</v>
+        <v>610</v>
       </c>
     </row>
     <row r="9">
@@ -898,18 +898,18 @@
       </c>
       <c r="G9" t="inlineStr"/>
       <c r="H9" t="n">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>Hrafnkell</t>
+          <t xml:space="preserve">Katrín Sig </t>
         </is>
       </c>
       <c r="J9" t="n">
         <v>2</v>
       </c>
       <c r="K9" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="L9" t="n">
         <v>3.5</v>
@@ -950,18 +950,18 @@
       </c>
       <c r="G10" t="inlineStr"/>
       <c r="H10" t="n">
-        <v>17</v>
+        <v>22</v>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Jórunn  </t>
+          <t xml:space="preserve">Magnús  </t>
         </is>
       </c>
       <c r="J10" t="n">
         <v>2</v>
       </c>
       <c r="K10" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="L10" t="n">
         <v>3.5</v>
@@ -970,7 +970,7 @@
         <v>70</v>
       </c>
       <c r="N10" t="n">
-        <v>640</v>
+        <v>660</v>
       </c>
     </row>
     <row r="11">
@@ -1002,18 +1002,18 @@
       </c>
       <c r="G11" t="inlineStr"/>
       <c r="H11" t="n">
-        <v>19</v>
+        <v>26</v>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t xml:space="preserve">Katrín Sig </t>
+          <t xml:space="preserve">Rut </t>
         </is>
       </c>
       <c r="J11" t="n">
         <v>2</v>
       </c>
       <c r="K11" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="L11" t="n">
         <v>3.5</v>
@@ -1022,7 +1022,7 @@
         <v>70</v>
       </c>
       <c r="N11" t="n">
-        <v>640</v>
+        <v>610</v>
       </c>
     </row>
     <row r="12">
@@ -1054,18 +1054,18 @@
       </c>
       <c r="G12" t="inlineStr"/>
       <c r="H12" t="n">
-        <v>22</v>
+        <v>30</v>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Magnús  </t>
+          <t xml:space="preserve">Sigríður </t>
         </is>
       </c>
       <c r="J12" t="n">
         <v>2</v>
       </c>
       <c r="K12" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="L12" t="n">
         <v>3.5</v>
@@ -1074,7 +1074,7 @@
         <v>70</v>
       </c>
       <c r="N12" t="n">
-        <v>610</v>
+        <v>390</v>
       </c>
     </row>
     <row r="13">
@@ -1106,18 +1106,18 @@
       </c>
       <c r="G13" t="inlineStr"/>
       <c r="H13" t="n">
-        <v>26</v>
+        <v>31</v>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t xml:space="preserve">Rut </t>
+          <t>Sveinn</t>
         </is>
       </c>
       <c r="J13" t="n">
         <v>2</v>
       </c>
       <c r="K13" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="L13" t="n">
         <v>3.5</v>
@@ -1126,7 +1126,7 @@
         <v>70</v>
       </c>
       <c r="N13" t="n">
-        <v>640</v>
+        <v>620</v>
       </c>
     </row>
     <row r="14">
@@ -1158,18 +1158,18 @@
       </c>
       <c r="G14" t="inlineStr"/>
       <c r="H14" t="n">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sigríður </t>
+          <t xml:space="preserve">Sæmundur </t>
         </is>
       </c>
       <c r="J14" t="n">
         <v>2</v>
       </c>
       <c r="K14" t="n">
-        <v>1</v>
+        <v>11</v>
       </c>
       <c r="L14" t="n">
         <v>3.5</v>
@@ -1178,7 +1178,7 @@
         <v>70</v>
       </c>
       <c r="N14" t="n">
-        <v>390</v>
+        <v>652.3</v>
       </c>
     </row>
     <row r="15">
@@ -1334,7 +1334,7 @@
         <v>80</v>
       </c>
       <c r="N17" t="n">
-        <v>560</v>
+        <v>610</v>
       </c>
     </row>
     <row r="18">
@@ -1377,7 +1377,7 @@
         <v>2</v>
       </c>
       <c r="K18" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="L18" t="n">
         <v>3</v>
@@ -1386,7 +1386,7 @@
         <v>70</v>
       </c>
       <c r="N18" t="n">
-        <v>590</v>
+        <v>600</v>
       </c>
     </row>
     <row r="19">
@@ -1429,7 +1429,7 @@
         <v>2</v>
       </c>
       <c r="K19" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="L19" t="n">
         <v>3</v>
@@ -1522,18 +1522,18 @@
       </c>
       <c r="G21" t="inlineStr"/>
       <c r="H21" t="n">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>Gréta</t>
+          <t xml:space="preserve">Elmar </t>
         </is>
       </c>
       <c r="J21" t="n">
         <v>2</v>
       </c>
       <c r="K21" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="L21" t="n">
         <v>3</v>
@@ -1542,7 +1542,7 @@
         <v>70</v>
       </c>
       <c r="N21" t="n">
-        <v>610</v>
+        <v>612.3</v>
       </c>
     </row>
     <row r="22">
@@ -1574,18 +1574,18 @@
       </c>
       <c r="G22" t="inlineStr"/>
       <c r="H22" t="n">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t xml:space="preserve">Guðný  </t>
+          <t>Hrafnkell</t>
         </is>
       </c>
       <c r="J22" t="n">
         <v>2</v>
       </c>
       <c r="K22" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="L22" t="n">
         <v>3</v>
@@ -1594,7 +1594,7 @@
         <v>70</v>
       </c>
       <c r="N22" t="n">
-        <v>600</v>
+        <v>410</v>
       </c>
     </row>
     <row r="23">
@@ -1626,18 +1626,18 @@
       </c>
       <c r="G23" t="inlineStr"/>
       <c r="H23" t="n">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>Hrafnkell</t>
+          <t xml:space="preserve">Laufey </t>
         </is>
       </c>
       <c r="J23" t="n">
         <v>2</v>
       </c>
       <c r="K23" t="n">
-        <v>3</v>
+        <v>11</v>
       </c>
       <c r="L23" t="n">
         <v>3</v>
@@ -1646,7 +1646,7 @@
         <v>70</v>
       </c>
       <c r="N23" t="n">
-        <v>410</v>
+        <v>640</v>
       </c>
     </row>
     <row r="24">
@@ -1741,7 +1741,7 @@
         <v>2</v>
       </c>
       <c r="K25" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="L25" t="n">
         <v>3</v>
@@ -1793,7 +1793,7 @@
         <v>2</v>
       </c>
       <c r="K26" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="L26" t="n">
         <v>3</v>
@@ -1897,7 +1897,7 @@
         <v>2</v>
       </c>
       <c r="K28" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="L28" t="n">
         <v>3</v>
@@ -1906,7 +1906,7 @@
         <v>70</v>
       </c>
       <c r="N28" t="n">
-        <v>640</v>
+        <v>580</v>
       </c>
     </row>
     <row r="29">
@@ -1958,7 +1958,7 @@
         <v>70</v>
       </c>
       <c r="N29" t="n">
-        <v>490</v>
+        <v>590</v>
       </c>
     </row>
     <row r="30">
@@ -2010,7 +2010,7 @@
         <v>70</v>
       </c>
       <c r="N30" t="n">
-        <v>560</v>
+        <v>520</v>
       </c>
     </row>
     <row r="31">
@@ -2114,7 +2114,7 @@
         <v>70</v>
       </c>
       <c r="N32" t="n">
-        <v>580</v>
+        <v>540</v>
       </c>
     </row>
     <row r="33">
@@ -2354,11 +2354,11 @@
       </c>
       <c r="G37" t="inlineStr"/>
       <c r="H37" t="n">
-        <v>24</v>
+        <v>31</v>
       </c>
       <c r="I37" t="inlineStr">
         <is>
-          <t>Orri</t>
+          <t>Sveinn</t>
         </is>
       </c>
       <c r="J37" t="n">
@@ -2374,7 +2374,7 @@
         <v>90</v>
       </c>
       <c r="N37" t="n">
-        <v>510</v>
+        <v>500</v>
       </c>
     </row>
     <row r="38">
@@ -2406,18 +2406,18 @@
       </c>
       <c r="G38" t="inlineStr"/>
       <c r="H38" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="I38" t="inlineStr">
         <is>
-          <t xml:space="preserve">Alda/ Miðó </t>
+          <t>Arnar Ragn</t>
         </is>
       </c>
       <c r="J38" t="n">
         <v>2</v>
       </c>
       <c r="K38" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="L38" t="n">
         <v>3.5</v>
@@ -2426,7 +2426,7 @@
         <v>50</v>
       </c>
       <c r="N38" t="n">
-        <v>510</v>
+        <v>460</v>
       </c>
     </row>
     <row r="39">
@@ -2458,18 +2458,18 @@
       </c>
       <c r="G39" t="inlineStr"/>
       <c r="H39" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="I39" t="inlineStr">
         <is>
-          <t>Arnar Ragn</t>
+          <t xml:space="preserve">Elísabet </t>
         </is>
       </c>
       <c r="J39" t="n">
         <v>2</v>
       </c>
       <c r="K39" t="n">
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="L39" t="n">
         <v>3.5</v>
@@ -2478,7 +2478,7 @@
         <v>50</v>
       </c>
       <c r="N39" t="n">
-        <v>460</v>
+        <v>660</v>
       </c>
     </row>
     <row r="40">
@@ -2510,18 +2510,18 @@
       </c>
       <c r="G40" t="inlineStr"/>
       <c r="H40" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="I40" t="inlineStr">
         <is>
-          <t xml:space="preserve">Elísabet </t>
+          <t xml:space="preserve">Erna </t>
         </is>
       </c>
       <c r="J40" t="n">
         <v>2</v>
       </c>
       <c r="K40" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="L40" t="n">
         <v>3.5</v>
@@ -2573,7 +2573,7 @@
         <v>2</v>
       </c>
       <c r="K41" t="n">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="L41" t="n">
         <v>3.5</v>
@@ -2582,7 +2582,7 @@
         <v>50</v>
       </c>
       <c r="N41" t="n">
-        <v>660</v>
+        <v>630</v>
       </c>
     </row>
     <row r="42">
@@ -2634,7 +2634,7 @@
         <v>50</v>
       </c>
       <c r="N42" t="n">
-        <v>650</v>
+        <v>630</v>
       </c>
     </row>
     <row r="43">
@@ -2677,7 +2677,7 @@
         <v>2</v>
       </c>
       <c r="K43" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="L43" t="n">
         <v>3.5</v>
@@ -2686,7 +2686,7 @@
         <v>50</v>
       </c>
       <c r="N43" t="n">
-        <v>530</v>
+        <v>540</v>
       </c>
     </row>
     <row r="44">
@@ -2718,18 +2718,18 @@
       </c>
       <c r="G44" t="inlineStr"/>
       <c r="H44" t="n">
-        <v>22</v>
+        <v>17</v>
       </c>
       <c r="I44" t="inlineStr">
         <is>
-          <t xml:space="preserve">Magnús  </t>
+          <t xml:space="preserve">Jórunn  </t>
         </is>
       </c>
       <c r="J44" t="n">
         <v>2</v>
       </c>
       <c r="K44" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L44" t="n">
         <v>3.5</v>
@@ -2738,7 +2738,7 @@
         <v>50</v>
       </c>
       <c r="N44" t="n">
-        <v>460</v>
+        <v>490</v>
       </c>
     </row>
     <row r="45">
@@ -2770,18 +2770,18 @@
       </c>
       <c r="G45" t="inlineStr"/>
       <c r="H45" t="n">
-        <v>27</v>
+        <v>19</v>
       </c>
       <c r="I45" t="inlineStr">
         <is>
-          <t>Sara B</t>
+          <t xml:space="preserve">Katrín Sig </t>
         </is>
       </c>
       <c r="J45" t="n">
         <v>2</v>
       </c>
       <c r="K45" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="L45" t="n">
         <v>3.5</v>
@@ -2790,7 +2790,7 @@
         <v>50</v>
       </c>
       <c r="N45" t="n">
-        <v>540</v>
+        <v>490</v>
       </c>
     </row>
     <row r="46">
@@ -2822,18 +2822,18 @@
       </c>
       <c r="G46" t="inlineStr"/>
       <c r="H46" t="n">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="I46" t="inlineStr">
         <is>
-          <t>Sveinn</t>
+          <t xml:space="preserve">Védís </t>
         </is>
       </c>
       <c r="J46" t="n">
         <v>2</v>
       </c>
       <c r="K46" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="L46" t="n">
         <v>3.5</v>
@@ -2842,7 +2842,7 @@
         <v>50</v>
       </c>
       <c r="N46" t="n">
-        <v>460</v>
+        <v>650</v>
       </c>
     </row>
     <row r="47">
@@ -2874,11 +2874,11 @@
       </c>
       <c r="G47" t="inlineStr"/>
       <c r="H47" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="I47" t="inlineStr">
         <is>
-          <t xml:space="preserve">Védís </t>
+          <t xml:space="preserve">Unnar </t>
         </is>
       </c>
       <c r="J47" t="n">
@@ -2894,7 +2894,7 @@
         <v>50</v>
       </c>
       <c r="N47" t="n">
-        <v>650</v>
+        <v>630</v>
       </c>
     </row>
     <row r="48">
@@ -2926,11 +2926,11 @@
       </c>
       <c r="G48" t="inlineStr"/>
       <c r="H48" t="n">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="I48" t="inlineStr">
         <is>
-          <t xml:space="preserve">Þórey </t>
+          <t xml:space="preserve">Róbert </t>
         </is>
       </c>
       <c r="J48" t="n">
@@ -2946,7 +2946,7 @@
         <v>50</v>
       </c>
       <c r="N48" t="n">
-        <v>540</v>
+        <v>520</v>
       </c>
     </row>
     <row r="49">
@@ -2978,18 +2978,18 @@
       </c>
       <c r="G49" t="inlineStr"/>
       <c r="H49" t="n">
-        <v>15</v>
+        <v>3</v>
       </c>
       <c r="I49" t="inlineStr">
         <is>
-          <t>Hrafnkell</t>
+          <t xml:space="preserve">Anna Soffía </t>
         </is>
       </c>
       <c r="J49" t="n">
         <v>2</v>
       </c>
       <c r="K49" t="n">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="L49" t="n">
         <v>3.5</v>
@@ -2998,7 +2998,7 @@
         <v>50</v>
       </c>
       <c r="N49" t="n">
-        <v>710</v>
+        <v>650</v>
       </c>
     </row>
     <row r="50">
@@ -3030,18 +3030,18 @@
       </c>
       <c r="G50" t="inlineStr"/>
       <c r="H50" t="n">
-        <v>20</v>
+        <v>9</v>
       </c>
       <c r="I50" t="inlineStr">
         <is>
-          <t xml:space="preserve">Laufey </t>
+          <t xml:space="preserve">Elmar </t>
         </is>
       </c>
       <c r="J50" t="n">
         <v>2</v>
       </c>
       <c r="K50" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="L50" t="n">
         <v>3.5</v>
@@ -3050,7 +3050,7 @@
         <v>50</v>
       </c>
       <c r="N50" t="n">
-        <v>630</v>
+        <v>462.3</v>
       </c>
     </row>
     <row r="51">
@@ -3082,18 +3082,18 @@
       </c>
       <c r="G51" t="inlineStr"/>
       <c r="H51" t="n">
-        <v>23</v>
+        <v>13</v>
       </c>
       <c r="I51" t="inlineStr">
         <is>
-          <t>Margrét Lára</t>
+          <t xml:space="preserve">Guðný  </t>
         </is>
       </c>
       <c r="J51" t="n">
         <v>2</v>
       </c>
       <c r="K51" t="n">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="L51" t="n">
         <v>3.5</v>
@@ -3102,7 +3102,7 @@
         <v>50</v>
       </c>
       <c r="N51" t="n">
-        <v>462.3</v>
+        <v>680</v>
       </c>
     </row>
     <row r="52">
@@ -3134,18 +3134,18 @@
       </c>
       <c r="G52" t="inlineStr"/>
       <c r="H52" t="n">
-        <v>28</v>
+        <v>20</v>
       </c>
       <c r="I52" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sara Júlía </t>
+          <t xml:space="preserve">Laufey </t>
         </is>
       </c>
       <c r="J52" t="n">
         <v>2</v>
       </c>
       <c r="K52" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="L52" t="n">
         <v>3.5</v>
@@ -3154,7 +3154,7 @@
         <v>50</v>
       </c>
       <c r="N52" t="n">
-        <v>510</v>
+        <v>490</v>
       </c>
     </row>
     <row r="53">
@@ -3186,18 +3186,18 @@
       </c>
       <c r="G53" t="inlineStr"/>
       <c r="H53" t="n">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="I53" t="inlineStr">
         <is>
-          <t xml:space="preserve">Selma </t>
+          <t xml:space="preserve">Rut </t>
         </is>
       </c>
       <c r="J53" t="n">
         <v>2</v>
       </c>
       <c r="K53" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="L53" t="n">
         <v>3.5</v>
@@ -3206,7 +3206,7 @@
         <v>50</v>
       </c>
       <c r="N53" t="n">
-        <v>530</v>
+        <v>490</v>
       </c>
     </row>
     <row r="54">
@@ -3238,18 +3238,18 @@
       </c>
       <c r="G54" t="inlineStr"/>
       <c r="H54" t="n">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="I54" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sigríður </t>
+          <t xml:space="preserve">Sæmundur </t>
         </is>
       </c>
       <c r="J54" t="n">
         <v>2</v>
       </c>
       <c r="K54" t="n">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="L54" t="n">
         <v>3.5</v>
@@ -3258,7 +3258,7 @@
         <v>50</v>
       </c>
       <c r="N54" t="n">
-        <v>700</v>
+        <v>702.3</v>
       </c>
     </row>
     <row r="55">
@@ -3290,18 +3290,18 @@
       </c>
       <c r="G55" t="inlineStr"/>
       <c r="H55" t="n">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="I55" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sæmundur </t>
+          <t xml:space="preserve">Védís </t>
         </is>
       </c>
       <c r="J55" t="n">
         <v>2</v>
       </c>
       <c r="K55" t="n">
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="L55" t="n">
         <v>3.5</v>
@@ -3310,7 +3310,7 @@
         <v>50</v>
       </c>
       <c r="N55" t="n">
-        <v>462.3</v>
+        <v>700</v>
       </c>
     </row>
     <row r="56">
@@ -3342,18 +3342,18 @@
       </c>
       <c r="G56" t="inlineStr"/>
       <c r="H56" t="n">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="I56" t="inlineStr">
         <is>
-          <t xml:space="preserve">Valdís </t>
+          <t xml:space="preserve">Unnar </t>
         </is>
       </c>
       <c r="J56" t="n">
         <v>2</v>
       </c>
       <c r="K56" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="L56" t="n">
         <v>3.5</v>
@@ -3362,7 +3362,7 @@
         <v>50</v>
       </c>
       <c r="N56" t="n">
-        <v>470</v>
+        <v>680</v>
       </c>
     </row>
     <row r="57">
@@ -3394,18 +3394,18 @@
       </c>
       <c r="G57" t="inlineStr"/>
       <c r="H57" t="n">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="I57" t="inlineStr">
         <is>
-          <t xml:space="preserve">Védís </t>
+          <t>Ömmi</t>
         </is>
       </c>
       <c r="J57" t="n">
         <v>2</v>
       </c>
       <c r="K57" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="L57" t="n">
         <v>3.5</v>
@@ -3414,7 +3414,7 @@
         <v>50</v>
       </c>
       <c r="N57" t="n">
-        <v>700</v>
+        <v>630</v>
       </c>
     </row>
     <row r="58">
@@ -3446,18 +3446,18 @@
       </c>
       <c r="G58" t="inlineStr"/>
       <c r="H58" t="n">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="I58" t="inlineStr">
         <is>
-          <t>Ömmi</t>
+          <t xml:space="preserve">Arnar </t>
         </is>
       </c>
       <c r="J58" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K58" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="L58" t="n">
         <v>3.5</v>
@@ -3466,7 +3466,7 @@
         <v>50</v>
       </c>
       <c r="N58" t="n">
-        <v>690</v>
+        <v>700</v>
       </c>
     </row>
     <row r="59">
@@ -3498,11 +3498,11 @@
       </c>
       <c r="G59" t="inlineStr"/>
       <c r="H59" t="n">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="I59" t="inlineStr">
         <is>
-          <t xml:space="preserve">Arnar </t>
+          <t xml:space="preserve">Þórey </t>
         </is>
       </c>
       <c r="J59" t="n">
@@ -3518,7 +3518,7 @@
         <v>50</v>
       </c>
       <c r="N59" t="n">
-        <v>610</v>
+        <v>640</v>
       </c>
     </row>
     <row r="60">
@@ -3550,11 +3550,11 @@
       </c>
       <c r="G60" t="inlineStr"/>
       <c r="H60" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I60" t="inlineStr">
         <is>
-          <t xml:space="preserve">Anna Soffía </t>
+          <t xml:space="preserve">Alda/ Miðó </t>
         </is>
       </c>
       <c r="J60" t="n">
@@ -3570,7 +3570,7 @@
         <v>50</v>
       </c>
       <c r="N60" t="n">
-        <v>450</v>
+        <v>460</v>
       </c>
     </row>
     <row r="61">
@@ -3706,18 +3706,18 @@
       </c>
       <c r="G63" t="inlineStr"/>
       <c r="H63" t="n">
-        <v>9</v>
+        <v>15</v>
       </c>
       <c r="I63" t="inlineStr">
         <is>
-          <t xml:space="preserve">Elmar </t>
+          <t>Hrafnkell</t>
         </is>
       </c>
       <c r="J63" t="n">
         <v>2</v>
       </c>
       <c r="K63" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="L63" t="n">
         <v>4</v>
@@ -3726,7 +3726,7 @@
         <v>50</v>
       </c>
       <c r="N63" t="n">
-        <v>462.3</v>
+        <v>710</v>
       </c>
     </row>
     <row r="64">
@@ -3758,18 +3758,18 @@
       </c>
       <c r="G64" t="inlineStr"/>
       <c r="H64" t="n">
-        <v>10</v>
+        <v>17</v>
       </c>
       <c r="I64" t="inlineStr">
         <is>
-          <t xml:space="preserve">Erna </t>
+          <t xml:space="preserve">Jórunn  </t>
         </is>
       </c>
       <c r="J64" t="n">
         <v>2</v>
       </c>
       <c r="K64" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="L64" t="n">
         <v>4</v>
@@ -3810,18 +3810,18 @@
       </c>
       <c r="G65" t="inlineStr"/>
       <c r="H65" t="n">
-        <v>12</v>
+        <v>19</v>
       </c>
       <c r="I65" t="inlineStr">
         <is>
-          <t>Gréta</t>
+          <t xml:space="preserve">Katrín Sig </t>
         </is>
       </c>
       <c r="J65" t="n">
         <v>2</v>
       </c>
       <c r="K65" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="L65" t="n">
         <v>4</v>
@@ -3862,18 +3862,18 @@
       </c>
       <c r="G66" t="inlineStr"/>
       <c r="H66" t="n">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="I66" t="inlineStr">
         <is>
-          <t xml:space="preserve">Magnús  </t>
+          <t xml:space="preserve">Laufey </t>
         </is>
       </c>
       <c r="J66" t="n">
         <v>2</v>
       </c>
       <c r="K66" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="L66" t="n">
         <v>4</v>
@@ -3882,7 +3882,7 @@
         <v>50</v>
       </c>
       <c r="N66" t="n">
-        <v>710</v>
+        <v>690</v>
       </c>
     </row>
     <row r="67">
@@ -3925,7 +3925,7 @@
         <v>2</v>
       </c>
       <c r="K67" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="L67" t="n">
         <v>4</v>
@@ -3934,7 +3934,7 @@
         <v>50</v>
       </c>
       <c r="N67" t="n">
-        <v>490</v>
+        <v>710</v>
       </c>
     </row>
     <row r="68">
@@ -3966,18 +3966,18 @@
       </c>
       <c r="G68" t="inlineStr"/>
       <c r="H68" t="n">
-        <v>32</v>
+        <v>27</v>
       </c>
       <c r="I68" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sæmundur </t>
+          <t>Sara B</t>
         </is>
       </c>
       <c r="J68" t="n">
         <v>2</v>
       </c>
       <c r="K68" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="L68" t="n">
         <v>4</v>
@@ -3986,7 +3986,7 @@
         <v>50</v>
       </c>
       <c r="N68" t="n">
-        <v>692.3</v>
+        <v>490</v>
       </c>
     </row>
     <row r="69">
@@ -4018,18 +4018,18 @@
       </c>
       <c r="G69" t="inlineStr"/>
       <c r="H69" t="n">
-        <v>33</v>
+        <v>28</v>
       </c>
       <c r="I69" t="inlineStr">
         <is>
-          <t xml:space="preserve">Valdís </t>
+          <t xml:space="preserve">Sara Júlía </t>
         </is>
       </c>
       <c r="J69" t="n">
         <v>2</v>
       </c>
       <c r="K69" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="L69" t="n">
         <v>4</v>
@@ -4038,7 +4038,7 @@
         <v>50</v>
       </c>
       <c r="N69" t="n">
-        <v>700</v>
+        <v>460</v>
       </c>
     </row>
     <row r="70">
@@ -4070,11 +4070,11 @@
       </c>
       <c r="G70" t="inlineStr"/>
       <c r="H70" t="n">
-        <v>36</v>
+        <v>31</v>
       </c>
       <c r="I70" t="inlineStr">
         <is>
-          <t xml:space="preserve">Unnar </t>
+          <t>Sveinn</t>
         </is>
       </c>
       <c r="J70" t="n">
@@ -4122,11 +4122,11 @@
       </c>
       <c r="G71" t="inlineStr"/>
       <c r="H71" t="n">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="I71" t="inlineStr">
         <is>
-          <t xml:space="preserve">Róbert </t>
+          <t xml:space="preserve">Þórey </t>
         </is>
       </c>
       <c r="J71" t="n">
@@ -4142,7 +4142,7 @@
         <v>50</v>
       </c>
       <c r="N71" t="n">
-        <v>590</v>
+        <v>690</v>
       </c>
     </row>
     <row r="72">
@@ -4174,18 +4174,18 @@
       </c>
       <c r="G72" t="inlineStr"/>
       <c r="H72" t="n">
-        <v>23</v>
+        <v>30</v>
       </c>
       <c r="I72" t="inlineStr">
         <is>
-          <t>Margrét Lára</t>
+          <t xml:space="preserve">Sigríður </t>
         </is>
       </c>
       <c r="J72" t="n">
         <v>2</v>
       </c>
       <c r="K72" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L72" t="n">
         <v>5</v>
@@ -4194,7 +4194,7 @@
         <v>60</v>
       </c>
       <c r="N72" t="n">
-        <v>522.3</v>
+        <v>450</v>
       </c>
     </row>
     <row r="73">
@@ -4226,18 +4226,18 @@
       </c>
       <c r="G73" t="inlineStr"/>
       <c r="H73" t="n">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="I73" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sigríður </t>
+          <t xml:space="preserve">Valdís </t>
         </is>
       </c>
       <c r="J73" t="n">
         <v>2</v>
       </c>
       <c r="K73" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L73" t="n">
         <v>5</v>
@@ -4246,7 +4246,7 @@
         <v>60</v>
       </c>
       <c r="N73" t="n">
-        <v>450</v>
+        <v>480</v>
       </c>
     </row>
     <row r="74">
@@ -4278,11 +4278,11 @@
       </c>
       <c r="G74" t="inlineStr"/>
       <c r="H74" t="n">
-        <v>20</v>
+        <v>29</v>
       </c>
       <c r="I74" t="inlineStr">
         <is>
-          <t xml:space="preserve">Laufey </t>
+          <t xml:space="preserve">Selma </t>
         </is>
       </c>
       <c r="J74" t="n">
@@ -4298,7 +4298,7 @@
         <v>40</v>
       </c>
       <c r="N74" t="n">
-        <v>480</v>
+        <v>470</v>
       </c>
     </row>
     <row r="75">
@@ -4330,11 +4330,11 @@
       </c>
       <c r="G75" t="inlineStr"/>
       <c r="H75" t="n">
-        <v>17</v>
+        <v>23</v>
       </c>
       <c r="I75" t="inlineStr">
         <is>
-          <t xml:space="preserve">Jórunn  </t>
+          <t>Margrét Lára</t>
         </is>
       </c>
       <c r="J75" t="n">
@@ -4350,7 +4350,7 @@
         <v>80</v>
       </c>
       <c r="N75" t="n">
-        <v>570</v>
+        <v>572.3</v>
       </c>
     </row>
     <row r="76">
@@ -4382,11 +4382,11 @@
       </c>
       <c r="G76" t="inlineStr"/>
       <c r="H76" t="n">
-        <v>16</v>
+        <v>5</v>
       </c>
       <c r="I76" t="inlineStr">
         <is>
-          <t xml:space="preserve">Hrannar </t>
+          <t xml:space="preserve">Auður </t>
         </is>
       </c>
       <c r="J76" t="n">
@@ -4402,7 +4402,7 @@
         <v>40</v>
       </c>
       <c r="N76" t="n">
-        <v>480</v>
+        <v>440</v>
       </c>
     </row>
     <row r="77">
@@ -4434,11 +4434,11 @@
       </c>
       <c r="G77" t="inlineStr"/>
       <c r="H77" t="n">
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="I77" t="inlineStr">
         <is>
-          <t xml:space="preserve">Unnar </t>
+          <t xml:space="preserve">Sæmundur </t>
         </is>
       </c>
       <c r="J77" t="n">
@@ -4454,7 +4454,7 @@
         <v>90</v>
       </c>
       <c r="N77" t="n">
-        <v>540</v>
+        <v>502.3</v>
       </c>
     </row>
     <row r="78">
@@ -4486,11 +4486,11 @@
       </c>
       <c r="G78" t="inlineStr"/>
       <c r="H78" t="n">
-        <v>13</v>
+        <v>35</v>
       </c>
       <c r="I78" t="inlineStr">
         <is>
-          <t xml:space="preserve">Guðný  </t>
+          <t xml:space="preserve">Védís </t>
         </is>
       </c>
       <c r="J78" t="n">
@@ -4590,18 +4590,18 @@
       </c>
       <c r="G80" t="inlineStr"/>
       <c r="H80" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="I80" t="inlineStr">
         <is>
-          <t xml:space="preserve">Alda/ Miðó </t>
+          <t>Arnar Ragn</t>
         </is>
       </c>
       <c r="J80" t="n">
         <v>2</v>
       </c>
       <c r="K80" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="L80" t="n">
         <v>3</v>
@@ -4610,7 +4610,7 @@
         <v>50</v>
       </c>
       <c r="N80" t="n">
-        <v>460</v>
+        <v>660</v>
       </c>
     </row>
     <row r="81">
@@ -4642,18 +4642,18 @@
       </c>
       <c r="G81" t="inlineStr"/>
       <c r="H81" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="I81" t="inlineStr">
         <is>
-          <t>Arnar Ragn</t>
+          <t xml:space="preserve">Elmar </t>
         </is>
       </c>
       <c r="J81" t="n">
         <v>2</v>
       </c>
       <c r="K81" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="L81" t="n">
         <v>3</v>
@@ -4662,7 +4662,7 @@
         <v>50</v>
       </c>
       <c r="N81" t="n">
-        <v>660</v>
+        <v>662.3</v>
       </c>
     </row>
     <row r="82">
@@ -4694,18 +4694,18 @@
       </c>
       <c r="G82" t="inlineStr"/>
       <c r="H82" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="I82" t="inlineStr">
         <is>
-          <t xml:space="preserve">Auður </t>
+          <t xml:space="preserve">Erna </t>
         </is>
       </c>
       <c r="J82" t="n">
         <v>2</v>
       </c>
       <c r="K82" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="L82" t="n">
         <v>3</v>
@@ -4714,7 +4714,7 @@
         <v>50</v>
       </c>
       <c r="N82" t="n">
-        <v>450</v>
+        <v>710</v>
       </c>
     </row>
     <row r="83">
@@ -4746,18 +4746,18 @@
       </c>
       <c r="G83" t="inlineStr"/>
       <c r="H83" t="n">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="I83" t="inlineStr">
         <is>
-          <t>Hrafnkell</t>
+          <t>Gréta</t>
         </is>
       </c>
       <c r="J83" t="n">
         <v>2</v>
       </c>
       <c r="K83" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="L83" t="n">
         <v>3</v>
@@ -4766,7 +4766,7 @@
         <v>50</v>
       </c>
       <c r="N83" t="n">
-        <v>660</v>
+        <v>500</v>
       </c>
     </row>
     <row r="84">
@@ -4798,18 +4798,18 @@
       </c>
       <c r="G84" t="inlineStr"/>
       <c r="H84" t="n">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="I84" t="inlineStr">
         <is>
-          <t xml:space="preserve">Jórunn  </t>
+          <t xml:space="preserve">Guðný  </t>
         </is>
       </c>
       <c r="J84" t="n">
         <v>2</v>
       </c>
       <c r="K84" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="L84" t="n">
         <v>3</v>
@@ -4818,7 +4818,7 @@
         <v>50</v>
       </c>
       <c r="N84" t="n">
-        <v>690</v>
+        <v>500</v>
       </c>
     </row>
     <row r="85">
@@ -4850,18 +4850,18 @@
       </c>
       <c r="G85" t="inlineStr"/>
       <c r="H85" t="n">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="I85" t="inlineStr">
         <is>
-          <t xml:space="preserve">Katrín Sig </t>
+          <t>Hrafnkell</t>
         </is>
       </c>
       <c r="J85" t="n">
         <v>2</v>
       </c>
       <c r="K85" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="L85" t="n">
         <v>3</v>
@@ -4870,7 +4870,7 @@
         <v>50</v>
       </c>
       <c r="N85" t="n">
-        <v>690</v>
+        <v>660</v>
       </c>
     </row>
     <row r="86">
@@ -4922,7 +4922,7 @@
         <v>50</v>
       </c>
       <c r="N86" t="n">
-        <v>660</v>
+        <v>710</v>
       </c>
     </row>
     <row r="87">
@@ -4954,18 +4954,18 @@
       </c>
       <c r="G87" t="inlineStr"/>
       <c r="H87" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="I87" t="inlineStr">
         <is>
-          <t xml:space="preserve">Selma </t>
+          <t xml:space="preserve">Sigríður </t>
         </is>
       </c>
       <c r="J87" t="n">
         <v>2</v>
       </c>
       <c r="K87" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="L87" t="n">
         <v>3</v>
@@ -4974,7 +4974,7 @@
         <v>50</v>
       </c>
       <c r="N87" t="n">
-        <v>480</v>
+        <v>650</v>
       </c>
     </row>
     <row r="88">
@@ -5006,18 +5006,18 @@
       </c>
       <c r="G88" t="inlineStr"/>
       <c r="H88" t="n">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="I88" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sigríður </t>
+          <t>Sveinn</t>
         </is>
       </c>
       <c r="J88" t="n">
         <v>2</v>
       </c>
       <c r="K88" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="L88" t="n">
         <v>3</v>
@@ -5026,7 +5026,7 @@
         <v>50</v>
       </c>
       <c r="N88" t="n">
-        <v>650</v>
+        <v>670</v>
       </c>
     </row>
     <row r="89">
@@ -5058,18 +5058,18 @@
       </c>
       <c r="G89" t="inlineStr"/>
       <c r="H89" t="n">
-        <v>31</v>
+        <v>36</v>
       </c>
       <c r="I89" t="inlineStr">
         <is>
-          <t>Sveinn</t>
+          <t xml:space="preserve">Unnar </t>
         </is>
       </c>
       <c r="J89" t="n">
         <v>2</v>
       </c>
       <c r="K89" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="L89" t="n">
         <v>3</v>
@@ -5078,7 +5078,7 @@
         <v>50</v>
       </c>
       <c r="N89" t="n">
-        <v>640</v>
+        <v>500</v>
       </c>
     </row>
     <row r="90">
@@ -5130,7 +5130,7 @@
         <v>50</v>
       </c>
       <c r="N90" t="n">
-        <v>540</v>
+        <v>570</v>
       </c>
     </row>
     <row r="91">
@@ -5338,7 +5338,7 @@
         <v>70</v>
       </c>
       <c r="N94" t="n">
-        <v>672.3</v>
+        <v>642.3</v>
       </c>
     </row>
     <row r="95">
@@ -5474,18 +5474,18 @@
       </c>
       <c r="G97" t="inlineStr"/>
       <c r="H97" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I97" t="inlineStr">
         <is>
-          <t xml:space="preserve">Anna Soffía </t>
+          <t xml:space="preserve">Alda/ Miðó </t>
         </is>
       </c>
       <c r="J97" t="n">
         <v>2</v>
       </c>
       <c r="K97" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="L97" t="n">
         <v>5.5</v>
@@ -5494,7 +5494,7 @@
         <v>70</v>
       </c>
       <c r="N97" t="n">
-        <v>400</v>
+        <v>580</v>
       </c>
     </row>
     <row r="98">
@@ -5526,18 +5526,18 @@
       </c>
       <c r="G98" t="inlineStr"/>
       <c r="H98" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="I98" t="inlineStr">
         <is>
-          <t xml:space="preserve">Auður </t>
+          <t xml:space="preserve">Anna Soffía </t>
         </is>
       </c>
       <c r="J98" t="n">
         <v>2</v>
       </c>
       <c r="K98" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="L98" t="n">
         <v>5.5</v>
@@ -5546,7 +5546,7 @@
         <v>70</v>
       </c>
       <c r="N98" t="n">
-        <v>570</v>
+        <v>400</v>
       </c>
     </row>
     <row r="99">
@@ -5630,18 +5630,18 @@
       </c>
       <c r="G100" t="inlineStr"/>
       <c r="H100" t="n">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="I100" t="inlineStr">
         <is>
-          <t xml:space="preserve">Hólmfríður </t>
+          <t xml:space="preserve">Hrannar </t>
         </is>
       </c>
       <c r="J100" t="n">
         <v>2</v>
       </c>
       <c r="K100" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="L100" t="n">
         <v>5.5</v>
@@ -5650,7 +5650,7 @@
         <v>70</v>
       </c>
       <c r="N100" t="n">
-        <v>630</v>
+        <v>610</v>
       </c>
     </row>
     <row r="101">
@@ -5745,7 +5745,7 @@
         <v>2</v>
       </c>
       <c r="K102" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="L102" t="n">
         <v>5.5</v>
@@ -5754,7 +5754,7 @@
         <v>70</v>
       </c>
       <c r="N102" t="n">
-        <v>610</v>
+        <v>630</v>
       </c>
     </row>
     <row r="103">
@@ -5797,7 +5797,7 @@
         <v>2</v>
       </c>
       <c r="K103" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="L103" t="n">
         <v>5.5</v>
@@ -5806,7 +5806,7 @@
         <v>70</v>
       </c>
       <c r="N103" t="n">
-        <v>580</v>
+        <v>600</v>
       </c>
     </row>
     <row r="104">
@@ -5849,7 +5849,7 @@
         <v>2</v>
       </c>
       <c r="K104" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="L104" t="n">
         <v>5.5</v>
@@ -5858,7 +5858,7 @@
         <v>70</v>
       </c>
       <c r="N104" t="n">
-        <v>600</v>
+        <v>540</v>
       </c>
     </row>
     <row r="105">
@@ -5962,7 +5962,7 @@
         <v>70</v>
       </c>
       <c r="N106" t="n">
-        <v>420</v>
+        <v>470</v>
       </c>
     </row>
     <row r="107">
@@ -6046,11 +6046,11 @@
       </c>
       <c r="G108" t="inlineStr"/>
       <c r="H108" t="n">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="I108" t="inlineStr">
         <is>
-          <t xml:space="preserve">Elmar </t>
+          <t xml:space="preserve">Auður </t>
         </is>
       </c>
       <c r="J108" t="n">
@@ -6066,7 +6066,7 @@
         <v>70</v>
       </c>
       <c r="N108" t="n">
-        <v>682.3</v>
+        <v>560</v>
       </c>
     </row>
     <row r="109">
@@ -6098,11 +6098,11 @@
       </c>
       <c r="G109" t="inlineStr"/>
       <c r="H109" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="I109" t="inlineStr">
         <is>
-          <t xml:space="preserve">Guðný  </t>
+          <t>Gréta</t>
         </is>
       </c>
       <c r="J109" t="n">
@@ -6118,7 +6118,7 @@
         <v>70</v>
       </c>
       <c r="N109" t="n">
-        <v>720</v>
+        <v>700</v>
       </c>
     </row>
     <row r="110">
@@ -6150,18 +6150,18 @@
       </c>
       <c r="G110" t="inlineStr"/>
       <c r="H110" t="n">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="I110" t="inlineStr">
         <is>
-          <t xml:space="preserve">Hrannar </t>
+          <t xml:space="preserve">Hólmfríður </t>
         </is>
       </c>
       <c r="J110" t="n">
         <v>2</v>
       </c>
       <c r="K110" t="n">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="L110" t="n">
         <v>4</v>
@@ -6170,7 +6170,7 @@
         <v>70</v>
       </c>
       <c r="N110" t="n">
-        <v>440</v>
+        <v>590</v>
       </c>
     </row>
     <row r="111">
@@ -6202,18 +6202,18 @@
       </c>
       <c r="G111" t="inlineStr"/>
       <c r="H111" t="n">
-        <v>26</v>
+        <v>16</v>
       </c>
       <c r="I111" t="inlineStr">
         <is>
-          <t xml:space="preserve">Rut </t>
+          <t xml:space="preserve">Hrannar </t>
         </is>
       </c>
       <c r="J111" t="n">
         <v>2</v>
       </c>
       <c r="K111" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="L111" t="n">
         <v>4</v>
@@ -6222,7 +6222,7 @@
         <v>70</v>
       </c>
       <c r="N111" t="n">
-        <v>710</v>
+        <v>440</v>
       </c>
     </row>
     <row r="112">
@@ -6254,18 +6254,18 @@
       </c>
       <c r="G112" t="inlineStr"/>
       <c r="H112" t="n">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="I112" t="inlineStr">
         <is>
-          <t>Sara B</t>
+          <t>Margrét Lára</t>
         </is>
       </c>
       <c r="J112" t="n">
         <v>2</v>
       </c>
       <c r="K112" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="L112" t="n">
         <v>4</v>
@@ -6274,7 +6274,7 @@
         <v>70</v>
       </c>
       <c r="N112" t="n">
-        <v>440</v>
+        <v>712.3</v>
       </c>
     </row>
     <row r="113">
@@ -6306,18 +6306,18 @@
       </c>
       <c r="G113" t="inlineStr"/>
       <c r="H113" t="n">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="I113" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sara Júlía </t>
+          <t>Sara B</t>
         </is>
       </c>
       <c r="J113" t="n">
         <v>2</v>
       </c>
       <c r="K113" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="L113" t="n">
         <v>4</v>
@@ -6326,7 +6326,7 @@
         <v>70</v>
       </c>
       <c r="N113" t="n">
-        <v>410</v>
+        <v>440</v>
       </c>
     </row>
     <row r="114">
@@ -6358,18 +6358,18 @@
       </c>
       <c r="G114" t="inlineStr"/>
       <c r="H114" t="n">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="I114" t="inlineStr">
         <is>
-          <t>Sveinn</t>
+          <t xml:space="preserve">Sara Júlía </t>
         </is>
       </c>
       <c r="J114" t="n">
         <v>2</v>
       </c>
       <c r="K114" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="L114" t="n">
         <v>4</v>
@@ -6378,7 +6378,7 @@
         <v>70</v>
       </c>
       <c r="N114" t="n">
-        <v>710</v>
+        <v>410</v>
       </c>
     </row>
     <row r="115">
@@ -6410,18 +6410,18 @@
       </c>
       <c r="G115" t="inlineStr"/>
       <c r="H115" t="n">
-        <v>38</v>
+        <v>29</v>
       </c>
       <c r="I115" t="inlineStr">
         <is>
-          <t xml:space="preserve">Arnar </t>
+          <t xml:space="preserve">Selma </t>
         </is>
       </c>
       <c r="J115" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K115" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="L115" t="n">
         <v>4</v>
@@ -6430,7 +6430,7 @@
         <v>70</v>
       </c>
       <c r="N115" t="n">
-        <v>510</v>
+        <v>610</v>
       </c>
     </row>
     <row r="116">
@@ -6462,18 +6462,18 @@
       </c>
       <c r="G116" t="inlineStr"/>
       <c r="H116" t="n">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="I116" t="inlineStr">
         <is>
-          <t xml:space="preserve">Róbert </t>
+          <t xml:space="preserve">Arnar </t>
         </is>
       </c>
       <c r="J116" t="n">
         <v>1</v>
       </c>
       <c r="K116" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="L116" t="n">
         <v>4</v>
@@ -6482,7 +6482,7 @@
         <v>70</v>
       </c>
       <c r="N116" t="n">
-        <v>660</v>
+        <v>600</v>
       </c>
     </row>
     <row r="117">
@@ -6514,18 +6514,18 @@
       </c>
       <c r="G117" t="inlineStr"/>
       <c r="H117" t="n">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="I117" t="inlineStr">
         <is>
-          <t xml:space="preserve">Jara </t>
+          <t xml:space="preserve">Róbert </t>
         </is>
       </c>
       <c r="J117" t="n">
         <v>1</v>
       </c>
       <c r="K117" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="L117" t="n">
         <v>4</v>
@@ -6534,7 +6534,7 @@
         <v>70</v>
       </c>
       <c r="N117" t="n">
-        <v>470</v>
+        <v>640</v>
       </c>
     </row>
     <row r="118">
@@ -6566,18 +6566,18 @@
       </c>
       <c r="G118" t="inlineStr"/>
       <c r="H118" t="n">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="I118" t="inlineStr">
         <is>
-          <t xml:space="preserve">Þórey </t>
+          <t xml:space="preserve">Jara </t>
         </is>
       </c>
       <c r="J118" t="n">
         <v>1</v>
       </c>
       <c r="K118" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="L118" t="n">
         <v>4</v>
@@ -6586,7 +6586,7 @@
         <v>70</v>
       </c>
       <c r="N118" t="n">
-        <v>710</v>
+        <v>540</v>
       </c>
     </row>
     <row r="119">
@@ -6618,11 +6618,11 @@
       </c>
       <c r="G119" t="inlineStr"/>
       <c r="H119" t="n">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="I119" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sæmundur </t>
+          <t xml:space="preserve">Valdís </t>
         </is>
       </c>
       <c r="J119" t="n">
@@ -6638,7 +6638,7 @@
         <v>80</v>
       </c>
       <c r="N119" t="n">
-        <v>542.3</v>
+        <v>560</v>
       </c>
     </row>
     <row r="120">
@@ -6670,11 +6670,11 @@
       </c>
       <c r="G120" t="inlineStr"/>
       <c r="H120" t="n">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="I120" t="inlineStr">
         <is>
-          <t xml:space="preserve">Valdís </t>
+          <t xml:space="preserve">Unnar </t>
         </is>
       </c>
       <c r="J120" t="n">
@@ -6690,7 +6690,7 @@
         <v>80</v>
       </c>
       <c r="N120" t="n">
-        <v>550</v>
+        <v>580</v>
       </c>
     </row>
     <row r="121">
@@ -6774,11 +6774,11 @@
       </c>
       <c r="G122" t="inlineStr"/>
       <c r="H122" t="n">
-        <v>10</v>
+        <v>37</v>
       </c>
       <c r="I122" t="inlineStr">
         <is>
-          <t xml:space="preserve">Erna </t>
+          <t>Ömmi</t>
         </is>
       </c>
       <c r="J122" t="n">
@@ -6794,7 +6794,7 @@
         <v>40</v>
       </c>
       <c r="N122" t="n">
-        <v>480</v>
+        <v>430</v>
       </c>
     </row>
     <row r="123">
@@ -6826,15 +6826,15 @@
       </c>
       <c r="G123" t="inlineStr"/>
       <c r="H123" t="n">
-        <v>12</v>
+        <v>38</v>
       </c>
       <c r="I123" t="inlineStr">
         <is>
-          <t>Gréta</t>
+          <t xml:space="preserve">Arnar </t>
         </is>
       </c>
       <c r="J123" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K123" t="n">
         <v>0</v>
@@ -6846,7 +6846,7 @@
         <v>90</v>
       </c>
       <c r="N123" t="n">
-        <v>540</v>
+        <v>530</v>
       </c>
     </row>
     <row r="124">
@@ -6878,18 +6878,18 @@
       </c>
       <c r="G124" t="inlineStr"/>
       <c r="H124" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="I124" t="inlineStr">
         <is>
-          <t xml:space="preserve">Elmar </t>
+          <t xml:space="preserve">Anna Soffía </t>
         </is>
       </c>
       <c r="J124" t="n">
         <v>2</v>
       </c>
       <c r="K124" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L124" t="n">
         <v>3</v>
@@ -6898,7 +6898,7 @@
         <v>80</v>
       </c>
       <c r="N124" t="n">
-        <v>542.3</v>
+        <v>530</v>
       </c>
     </row>
     <row r="125">
@@ -6930,11 +6930,11 @@
       </c>
       <c r="G125" t="inlineStr"/>
       <c r="H125" t="n">
-        <v>23</v>
+        <v>12</v>
       </c>
       <c r="I125" t="inlineStr">
         <is>
-          <t>Margrét Lára</t>
+          <t>Gréta</t>
         </is>
       </c>
       <c r="J125" t="n">
@@ -6950,7 +6950,7 @@
         <v>80</v>
       </c>
       <c r="N125" t="n">
-        <v>602.3</v>
+        <v>580</v>
       </c>
     </row>
     <row r="126">
@@ -6982,11 +6982,11 @@
       </c>
       <c r="G126" t="inlineStr"/>
       <c r="H126" t="n">
-        <v>36</v>
+        <v>13</v>
       </c>
       <c r="I126" t="inlineStr">
         <is>
-          <t xml:space="preserve">Unnar </t>
+          <t xml:space="preserve">Guðný  </t>
         </is>
       </c>
       <c r="J126" t="n">
@@ -7002,7 +7002,7 @@
         <v>80</v>
       </c>
       <c r="N126" t="n">
-        <v>620</v>
+        <v>580</v>
       </c>
     </row>
     <row r="127">
@@ -7034,18 +7034,18 @@
       </c>
       <c r="G127" t="inlineStr"/>
       <c r="H127" t="n">
-        <v>37</v>
+        <v>20</v>
       </c>
       <c r="I127" t="inlineStr">
         <is>
-          <t>Ömmi</t>
+          <t xml:space="preserve">Laufey </t>
         </is>
       </c>
       <c r="J127" t="n">
         <v>2</v>
       </c>
       <c r="K127" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L127" t="n">
         <v>3</v>
@@ -7086,18 +7086,18 @@
       </c>
       <c r="G128" t="inlineStr"/>
       <c r="H128" t="n">
-        <v>2</v>
+        <v>11</v>
       </c>
       <c r="I128" t="inlineStr">
         <is>
-          <t xml:space="preserve">Alda/ Miðó </t>
+          <t xml:space="preserve">Gaukur </t>
         </is>
       </c>
       <c r="J128" t="n">
         <v>2</v>
       </c>
       <c r="K128" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="L128" t="n">
         <v>3</v>
@@ -7106,7 +7106,7 @@
         <v>50</v>
       </c>
       <c r="N128" t="n">
-        <v>560</v>
+        <v>520</v>
       </c>
     </row>
     <row r="129">
@@ -7138,18 +7138,18 @@
       </c>
       <c r="G129" t="inlineStr"/>
       <c r="H129" t="n">
-        <v>3</v>
+        <v>14</v>
       </c>
       <c r="I129" t="inlineStr">
         <is>
-          <t xml:space="preserve">Anna Soffía </t>
+          <t xml:space="preserve">Hólmfríður </t>
         </is>
       </c>
       <c r="J129" t="n">
         <v>2</v>
       </c>
       <c r="K129" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="L129" t="n">
         <v>3</v>
@@ -7158,7 +7158,7 @@
         <v>50</v>
       </c>
       <c r="N129" t="n">
-        <v>640</v>
+        <v>450</v>
       </c>
     </row>
     <row r="130">
@@ -7190,18 +7190,18 @@
       </c>
       <c r="G130" t="inlineStr"/>
       <c r="H130" t="n">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="I130" t="inlineStr">
         <is>
-          <t xml:space="preserve">Hrannar </t>
+          <t>Katrín Hel</t>
         </is>
       </c>
       <c r="J130" t="n">
         <v>2</v>
       </c>
       <c r="K130" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="L130" t="n">
         <v>3</v>
@@ -7210,7 +7210,7 @@
         <v>50</v>
       </c>
       <c r="N130" t="n">
-        <v>580</v>
+        <v>392.3</v>
       </c>
     </row>
     <row r="131">
@@ -7242,18 +7242,18 @@
       </c>
       <c r="G131" t="inlineStr"/>
       <c r="H131" t="n">
-        <v>18</v>
+        <v>24</v>
       </c>
       <c r="I131" t="inlineStr">
         <is>
-          <t>Katrín Hel</t>
+          <t>Orri</t>
         </is>
       </c>
       <c r="J131" t="n">
         <v>2</v>
       </c>
       <c r="K131" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="L131" t="n">
         <v>3</v>
@@ -7262,7 +7262,7 @@
         <v>50</v>
       </c>
       <c r="N131" t="n">
-        <v>392.3</v>
+        <v>470</v>
       </c>
     </row>
     <row r="132">
@@ -7294,18 +7294,18 @@
       </c>
       <c r="G132" t="inlineStr"/>
       <c r="H132" t="n">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="I132" t="inlineStr">
         <is>
-          <t>Sara B</t>
+          <t xml:space="preserve">Sigríður </t>
         </is>
       </c>
       <c r="J132" t="n">
         <v>2</v>
       </c>
       <c r="K132" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="L132" t="n">
         <v>3</v>
@@ -7314,7 +7314,7 @@
         <v>50</v>
       </c>
       <c r="N132" t="n">
-        <v>490</v>
+        <v>700</v>
       </c>
     </row>
     <row r="133">
@@ -7346,18 +7346,18 @@
       </c>
       <c r="G133" t="inlineStr"/>
       <c r="H133" t="n">
-        <v>28</v>
+        <v>33</v>
       </c>
       <c r="I133" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sara Júlía </t>
+          <t xml:space="preserve">Valdís </t>
         </is>
       </c>
       <c r="J133" t="n">
         <v>2</v>
       </c>
       <c r="K133" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="L133" t="n">
         <v>3</v>
@@ -7366,7 +7366,7 @@
         <v>50</v>
       </c>
       <c r="N133" t="n">
-        <v>460</v>
+        <v>730</v>
       </c>
     </row>
     <row r="134">
@@ -7398,11 +7398,11 @@
       </c>
       <c r="G134" t="inlineStr"/>
       <c r="H134" t="n">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="I134" t="inlineStr">
         <is>
-          <t xml:space="preserve">Þórey </t>
+          <t xml:space="preserve">Jara </t>
         </is>
       </c>
       <c r="J134" t="n">
@@ -7418,7 +7418,7 @@
         <v>50</v>
       </c>
       <c r="N134" t="n">
-        <v>590</v>
+        <v>470</v>
       </c>
     </row>
     <row r="135">
@@ -7502,11 +7502,11 @@
       </c>
       <c r="G136" t="inlineStr"/>
       <c r="H136" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="I136" t="inlineStr">
         <is>
-          <t xml:space="preserve">Magnús  </t>
+          <t>Margrét Lára</t>
         </is>
       </c>
       <c r="J136" t="n">
@@ -7522,7 +7522,7 @@
         <v>80</v>
       </c>
       <c r="N136" t="n">
-        <v>540</v>
+        <v>492.3</v>
       </c>
     </row>
     <row r="137">
@@ -7554,11 +7554,11 @@
       </c>
       <c r="G137" t="inlineStr"/>
       <c r="H137" t="n">
-        <v>11</v>
+        <v>22</v>
       </c>
       <c r="I137" t="inlineStr">
         <is>
-          <t xml:space="preserve">Gaukur </t>
+          <t xml:space="preserve">Magnús  </t>
         </is>
       </c>
       <c r="J137" t="n">
@@ -7574,7 +7574,7 @@
         <v>100</v>
       </c>
       <c r="N137" t="n">
-        <v>520</v>
+        <v>510</v>
       </c>
     </row>
     <row r="138">
@@ -7606,18 +7606,18 @@
       </c>
       <c r="G138" t="inlineStr"/>
       <c r="H138" t="n">
-        <v>19</v>
+        <v>9</v>
       </c>
       <c r="I138" t="inlineStr">
         <is>
-          <t xml:space="preserve">Katrín Sig </t>
+          <t xml:space="preserve">Elmar </t>
         </is>
       </c>
       <c r="J138" t="n">
         <v>2</v>
       </c>
       <c r="K138" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L138" t="n">
         <v>4</v>
@@ -7626,7 +7626,7 @@
         <v>80</v>
       </c>
       <c r="N138" t="n">
-        <v>570</v>
+        <v>542.3</v>
       </c>
     </row>
     <row r="139">
@@ -7658,18 +7658,18 @@
       </c>
       <c r="G139" t="inlineStr"/>
       <c r="H139" t="n">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="I139" t="inlineStr">
         <is>
-          <t xml:space="preserve">Rut </t>
+          <t xml:space="preserve">Sæmundur </t>
         </is>
       </c>
       <c r="J139" t="n">
         <v>2</v>
       </c>
       <c r="K139" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L139" t="n">
         <v>4</v>
@@ -7678,7 +7678,7 @@
         <v>80</v>
       </c>
       <c r="N139" t="n">
-        <v>570</v>
+        <v>582.3</v>
       </c>
     </row>
     <row r="140">
@@ -7762,18 +7762,18 @@
       </c>
       <c r="G141" t="inlineStr"/>
       <c r="H141" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="I141" t="inlineStr">
         <is>
-          <t xml:space="preserve">Erna </t>
+          <t xml:space="preserve">Gaukur </t>
         </is>
       </c>
       <c r="J141" t="n">
         <v>2</v>
       </c>
       <c r="K141" t="n">
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="L141" t="n">
         <v>4</v>
@@ -7782,7 +7782,7 @@
         <v>50</v>
       </c>
       <c r="N141" t="n">
-        <v>610</v>
+        <v>470</v>
       </c>
     </row>
     <row r="142">
@@ -7970,18 +7970,18 @@
       </c>
       <c r="G145" t="inlineStr"/>
       <c r="H145" t="n">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="I145" t="inlineStr">
         <is>
-          <t xml:space="preserve">Laufey </t>
+          <t xml:space="preserve">Jórunn  </t>
         </is>
       </c>
       <c r="J145" t="n">
         <v>2</v>
       </c>
       <c r="K145" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="L145" t="n">
         <v>4</v>
@@ -7990,7 +7990,7 @@
         <v>50</v>
       </c>
       <c r="N145" t="n">
-        <v>530</v>
+        <v>540</v>
       </c>
     </row>
     <row r="146">
@@ -8022,18 +8022,18 @@
       </c>
       <c r="G146" t="inlineStr"/>
       <c r="H146" t="n">
-        <v>31</v>
+        <v>19</v>
       </c>
       <c r="I146" t="inlineStr">
         <is>
-          <t>Sveinn</t>
+          <t xml:space="preserve">Katrín Sig </t>
         </is>
       </c>
       <c r="J146" t="n">
         <v>2</v>
       </c>
       <c r="K146" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="L146" t="n">
         <v>4</v>
@@ -8042,7 +8042,7 @@
         <v>50</v>
       </c>
       <c r="N146" t="n">
-        <v>590</v>
+        <v>540</v>
       </c>
     </row>
     <row r="147">
@@ -8074,18 +8074,18 @@
       </c>
       <c r="G147" t="inlineStr"/>
       <c r="H147" t="n">
-        <v>32</v>
+        <v>26</v>
       </c>
       <c r="I147" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sæmundur </t>
+          <t xml:space="preserve">Rut </t>
         </is>
       </c>
       <c r="J147" t="n">
         <v>2</v>
       </c>
       <c r="K147" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="L147" t="n">
         <v>4</v>
@@ -8094,7 +8094,7 @@
         <v>50</v>
       </c>
       <c r="N147" t="n">
-        <v>592.3</v>
+        <v>540</v>
       </c>
     </row>
     <row r="148">
@@ -8126,18 +8126,18 @@
       </c>
       <c r="G148" t="inlineStr"/>
       <c r="H148" t="n">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="I148" t="inlineStr">
         <is>
-          <t xml:space="preserve">Valdís </t>
+          <t>Sveinn</t>
         </is>
       </c>
       <c r="J148" t="n">
         <v>2</v>
       </c>
       <c r="K148" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="L148" t="n">
         <v>4</v>
@@ -8146,7 +8146,7 @@
         <v>50</v>
       </c>
       <c r="N148" t="n">
-        <v>600</v>
+        <v>550</v>
       </c>
     </row>
     <row r="149">
@@ -8282,11 +8282,11 @@
       </c>
       <c r="G151" t="inlineStr"/>
       <c r="H151" t="n">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="I151" t="inlineStr">
         <is>
-          <t xml:space="preserve">Jara </t>
+          <t xml:space="preserve">Róbert </t>
         </is>
       </c>
       <c r="J151" t="n">
@@ -8386,18 +8386,18 @@
       </c>
       <c r="G153" t="inlineStr"/>
       <c r="H153" t="n">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="I153" t="inlineStr">
         <is>
-          <t xml:space="preserve">Gaukur </t>
+          <t xml:space="preserve">Hólmfríður </t>
         </is>
       </c>
       <c r="J153" t="n">
         <v>2</v>
       </c>
       <c r="K153" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="L153" t="n">
         <v>4</v>
@@ -8406,7 +8406,7 @@
         <v>70</v>
       </c>
       <c r="N153" t="n">
-        <v>590</v>
+        <v>400</v>
       </c>
     </row>
     <row r="154">
@@ -8438,18 +8438,18 @@
       </c>
       <c r="G154" t="inlineStr"/>
       <c r="H154" t="n">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="I154" t="inlineStr">
         <is>
-          <t xml:space="preserve">Hólmfríður </t>
+          <t>Orri</t>
         </is>
       </c>
       <c r="J154" t="n">
         <v>2</v>
       </c>
       <c r="K154" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="L154" t="n">
         <v>4</v>
@@ -8458,7 +8458,7 @@
         <v>70</v>
       </c>
       <c r="N154" t="n">
-        <v>400</v>
+        <v>420</v>
       </c>
     </row>
     <row r="155">
@@ -8490,18 +8490,18 @@
       </c>
       <c r="G155" t="inlineStr"/>
       <c r="H155" t="n">
-        <v>18</v>
+        <v>27</v>
       </c>
       <c r="I155" t="inlineStr">
         <is>
-          <t>Katrín Hel</t>
+          <t>Sara B</t>
         </is>
       </c>
       <c r="J155" t="n">
         <v>2</v>
       </c>
       <c r="K155" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="L155" t="n">
         <v>4</v>
@@ -8510,7 +8510,7 @@
         <v>70</v>
       </c>
       <c r="N155" t="n">
-        <v>462.3</v>
+        <v>560</v>
       </c>
     </row>
     <row r="156">
@@ -8542,18 +8542,18 @@
       </c>
       <c r="G156" t="inlineStr"/>
       <c r="H156" t="n">
-        <v>24</v>
+        <v>28</v>
       </c>
       <c r="I156" t="inlineStr">
         <is>
-          <t>Orri</t>
+          <t xml:space="preserve">Sara Júlía </t>
         </is>
       </c>
       <c r="J156" t="n">
         <v>2</v>
       </c>
       <c r="K156" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="L156" t="n">
         <v>4</v>
@@ -8562,7 +8562,7 @@
         <v>70</v>
       </c>
       <c r="N156" t="n">
-        <v>420</v>
+        <v>530</v>
       </c>
     </row>
     <row r="157">
@@ -8646,18 +8646,18 @@
       </c>
       <c r="G158" t="inlineStr"/>
       <c r="H158" t="n">
-        <v>38</v>
+        <v>33</v>
       </c>
       <c r="I158" t="inlineStr">
         <is>
-          <t xml:space="preserve">Arnar </t>
+          <t xml:space="preserve">Valdís </t>
         </is>
       </c>
       <c r="J158" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K158" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="L158" t="n">
         <v>4</v>
@@ -8666,7 +8666,7 @@
         <v>70</v>
       </c>
       <c r="N158" t="n">
-        <v>680</v>
+        <v>630</v>
       </c>
     </row>
     <row r="159">
@@ -8698,11 +8698,11 @@
       </c>
       <c r="G159" t="inlineStr"/>
       <c r="H159" t="n">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="I159" t="inlineStr">
         <is>
-          <t xml:space="preserve">Róbert </t>
+          <t xml:space="preserve">Jara </t>
         </is>
       </c>
       <c r="J159" t="n">
@@ -8718,7 +8718,7 @@
         <v>70</v>
       </c>
       <c r="N159" t="n">
-        <v>490</v>
+        <v>420</v>
       </c>
     </row>
     <row r="160">
@@ -8761,7 +8761,7 @@
         <v>2</v>
       </c>
       <c r="K160" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L160" t="n">
         <v>3</v>
@@ -8802,18 +8802,18 @@
       </c>
       <c r="G161" t="inlineStr"/>
       <c r="H161" t="n">
-        <v>35</v>
+        <v>15</v>
       </c>
       <c r="I161" t="inlineStr">
         <is>
-          <t xml:space="preserve">Védís </t>
+          <t>Hrafnkell</t>
         </is>
       </c>
       <c r="J161" t="n">
         <v>2</v>
       </c>
       <c r="K161" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L161" t="n">
         <v>3</v>
@@ -8822,7 +8822,7 @@
         <v>80</v>
       </c>
       <c r="N161" t="n">
-        <v>530</v>
+        <v>540</v>
       </c>
     </row>
     <row r="162">
@@ -8854,11 +8854,11 @@
       </c>
       <c r="G162" t="inlineStr"/>
       <c r="H162" t="n">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="I162" t="inlineStr">
         <is>
-          <t xml:space="preserve">Hólmfríður </t>
+          <t xml:space="preserve">Erna </t>
         </is>
       </c>
       <c r="J162" t="n">
@@ -8874,7 +8874,7 @@
         <v>90</v>
       </c>
       <c r="N162" t="n">
-        <v>490</v>
+        <v>530</v>
       </c>
     </row>
     <row r="163">
@@ -8906,18 +8906,18 @@
       </c>
       <c r="G163" t="inlineStr"/>
       <c r="H163" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="I163" t="inlineStr">
         <is>
-          <t xml:space="preserve">Auður </t>
+          <t xml:space="preserve">Alda/ Miðó </t>
         </is>
       </c>
       <c r="J163" t="n">
         <v>2</v>
       </c>
       <c r="K163" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="L163" t="n">
         <v>3</v>
@@ -8926,7 +8926,7 @@
         <v>50</v>
       </c>
       <c r="N163" t="n">
-        <v>500</v>
+        <v>510</v>
       </c>
     </row>
     <row r="164">
@@ -8958,18 +8958,18 @@
       </c>
       <c r="G164" t="inlineStr"/>
       <c r="H164" t="n">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="I164" t="inlineStr">
         <is>
-          <t xml:space="preserve">Erna </t>
+          <t xml:space="preserve">Anna Soffía </t>
         </is>
       </c>
       <c r="J164" t="n">
         <v>2</v>
       </c>
       <c r="K164" t="n">
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="L164" t="n">
         <v>3</v>
@@ -8978,7 +8978,7 @@
         <v>50</v>
       </c>
       <c r="N164" t="n">
-        <v>660</v>
+        <v>450</v>
       </c>
     </row>
     <row r="165">
@@ -9010,18 +9010,18 @@
       </c>
       <c r="G165" t="inlineStr"/>
       <c r="H165" t="n">
-        <v>11</v>
+        <v>5</v>
       </c>
       <c r="I165" t="inlineStr">
         <is>
-          <t xml:space="preserve">Gaukur </t>
+          <t xml:space="preserve">Auður </t>
         </is>
       </c>
       <c r="J165" t="n">
         <v>2</v>
       </c>
       <c r="K165" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="L165" t="n">
         <v>3</v>
@@ -9030,7 +9030,7 @@
         <v>50</v>
       </c>
       <c r="N165" t="n">
-        <v>420</v>
+        <v>490</v>
       </c>
     </row>
     <row r="166">
@@ -9062,18 +9062,18 @@
       </c>
       <c r="G166" t="inlineStr"/>
       <c r="H166" t="n">
-        <v>17</v>
+        <v>11</v>
       </c>
       <c r="I166" t="inlineStr">
         <is>
-          <t xml:space="preserve">Jórunn  </t>
+          <t xml:space="preserve">Gaukur </t>
         </is>
       </c>
       <c r="J166" t="n">
         <v>2</v>
       </c>
       <c r="K166" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L166" t="n">
         <v>3</v>
@@ -9082,7 +9082,7 @@
         <v>50</v>
       </c>
       <c r="N166" t="n">
-        <v>490</v>
+        <v>420</v>
       </c>
     </row>
     <row r="167">
@@ -9114,11 +9114,11 @@
       </c>
       <c r="G167" t="inlineStr"/>
       <c r="H167" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="I167" t="inlineStr">
         <is>
-          <t xml:space="preserve">Katrín Sig </t>
+          <t xml:space="preserve">Hrannar </t>
         </is>
       </c>
       <c r="J167" t="n">
@@ -9166,18 +9166,18 @@
       </c>
       <c r="G168" t="inlineStr"/>
       <c r="H168" t="n">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="I168" t="inlineStr">
         <is>
-          <t xml:space="preserve">Laufey </t>
+          <t xml:space="preserve">Jórunn  </t>
         </is>
       </c>
       <c r="J168" t="n">
         <v>2</v>
       </c>
       <c r="K168" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="L168" t="n">
         <v>3</v>
@@ -9186,7 +9186,7 @@
         <v>50</v>
       </c>
       <c r="N168" t="n">
-        <v>580</v>
+        <v>660</v>
       </c>
     </row>
     <row r="169">
@@ -9218,18 +9218,18 @@
       </c>
       <c r="G169" t="inlineStr"/>
       <c r="H169" t="n">
-        <v>32</v>
+        <v>18</v>
       </c>
       <c r="I169" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sæmundur </t>
+          <t>Katrín Hel</t>
         </is>
       </c>
       <c r="J169" t="n">
         <v>2</v>
       </c>
       <c r="K169" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="L169" t="n">
         <v>3</v>
@@ -9238,7 +9238,7 @@
         <v>50</v>
       </c>
       <c r="N169" t="n">
-        <v>642.3</v>
+        <v>442.3</v>
       </c>
     </row>
     <row r="170">
@@ -9270,11 +9270,11 @@
       </c>
       <c r="G170" t="inlineStr"/>
       <c r="H170" t="n">
-        <v>33</v>
+        <v>19</v>
       </c>
       <c r="I170" t="inlineStr">
         <is>
-          <t xml:space="preserve">Valdís </t>
+          <t xml:space="preserve">Katrín Sig </t>
         </is>
       </c>
       <c r="J170" t="n">
@@ -9290,7 +9290,7 @@
         <v>50</v>
       </c>
       <c r="N170" t="n">
-        <v>650</v>
+        <v>660</v>
       </c>
     </row>
     <row r="171">
@@ -9322,18 +9322,18 @@
       </c>
       <c r="G171" t="inlineStr"/>
       <c r="H171" t="n">
-        <v>36</v>
+        <v>26</v>
       </c>
       <c r="I171" t="inlineStr">
         <is>
-          <t xml:space="preserve">Unnar </t>
+          <t xml:space="preserve">Rut </t>
         </is>
       </c>
       <c r="J171" t="n">
         <v>2</v>
       </c>
       <c r="K171" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="L171" t="n">
         <v>3</v>
@@ -9342,7 +9342,7 @@
         <v>50</v>
       </c>
       <c r="N171" t="n">
-        <v>670</v>
+        <v>660</v>
       </c>
     </row>
     <row r="172">
@@ -9374,18 +9374,18 @@
       </c>
       <c r="G172" t="inlineStr"/>
       <c r="H172" t="n">
-        <v>38</v>
+        <v>33</v>
       </c>
       <c r="I172" t="inlineStr">
         <is>
-          <t xml:space="preserve">Arnar </t>
+          <t xml:space="preserve">Valdís </t>
         </is>
       </c>
       <c r="J172" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K172" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="L172" t="n">
         <v>3</v>
@@ -9394,7 +9394,7 @@
         <v>50</v>
       </c>
       <c r="N172" t="n">
-        <v>560</v>
+        <v>680</v>
       </c>
     </row>
     <row r="173">
@@ -9426,18 +9426,18 @@
       </c>
       <c r="G173" t="inlineStr"/>
       <c r="H173" t="n">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="I173" t="inlineStr">
         <is>
-          <t xml:space="preserve">Þórey </t>
+          <t xml:space="preserve">Arnar </t>
         </is>
       </c>
       <c r="J173" t="n">
         <v>1</v>
       </c>
       <c r="K173" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="L173" t="n">
         <v>3</v>
@@ -9446,7 +9446,7 @@
         <v>50</v>
       </c>
       <c r="N173" t="n">
-        <v>640</v>
+        <v>650</v>
       </c>
     </row>
     <row r="174">
@@ -9478,11 +9478,11 @@
       </c>
       <c r="G174" t="inlineStr"/>
       <c r="H174" t="n">
-        <v>15</v>
+        <v>22</v>
       </c>
       <c r="I174" t="inlineStr">
         <is>
-          <t>Hrafnkell</t>
+          <t xml:space="preserve">Magnús  </t>
         </is>
       </c>
       <c r="J174" t="n">
@@ -9498,7 +9498,7 @@
         <v>80</v>
       </c>
       <c r="N174" t="n">
-        <v>540</v>
+        <v>590</v>
       </c>
     </row>
     <row r="175">
@@ -9530,11 +9530,11 @@
       </c>
       <c r="G175" t="inlineStr"/>
       <c r="H175" t="n">
-        <v>31</v>
+        <v>37</v>
       </c>
       <c r="I175" t="inlineStr">
         <is>
-          <t>Sveinn</t>
+          <t>Ömmi</t>
         </is>
       </c>
       <c r="J175" t="n">
@@ -9550,7 +9550,7 @@
         <v>80</v>
       </c>
       <c r="N175" t="n">
-        <v>540</v>
+        <v>510</v>
       </c>
     </row>
   </sheetData>
@@ -9771,20 +9771,20 @@
       <c r="G3" t="inlineStr"/>
       <c r="H3" t="inlineStr"/>
       <c r="I3" t="inlineStr"/>
-      <c r="J3" t="n">
-        <v>1</v>
-      </c>
+      <c r="J3" t="inlineStr"/>
       <c r="K3" t="inlineStr"/>
-      <c r="L3" t="inlineStr"/>
+      <c r="L3" t="n">
+        <v>1</v>
+      </c>
       <c r="M3" t="inlineStr"/>
       <c r="N3" t="inlineStr"/>
       <c r="O3" t="inlineStr"/>
       <c r="P3" t="inlineStr"/>
-      <c r="Q3" t="n">
-        <v>1</v>
-      </c>
+      <c r="Q3" t="inlineStr"/>
       <c r="R3" t="inlineStr"/>
-      <c r="S3" t="inlineStr"/>
+      <c r="S3" t="n">
+        <v>1</v>
+      </c>
       <c r="T3" t="n">
         <v>1</v>
       </c>
@@ -9792,23 +9792,21 @@
       <c r="V3" t="inlineStr"/>
       <c r="W3" t="inlineStr"/>
       <c r="X3" t="inlineStr"/>
-      <c r="Y3" t="n">
-        <v>1</v>
-      </c>
+      <c r="Y3" t="inlineStr"/>
       <c r="Z3" t="inlineStr"/>
       <c r="AA3" t="inlineStr"/>
       <c r="AB3" t="inlineStr"/>
       <c r="AC3" t="inlineStr"/>
       <c r="AD3" t="inlineStr"/>
-      <c r="AE3" t="inlineStr"/>
+      <c r="AE3" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
         <v>3</v>
       </c>
-      <c r="B4" t="n">
-        <v>1</v>
-      </c>
+      <c r="B4" t="inlineStr"/>
       <c r="C4" t="n">
         <v>1</v>
       </c>
@@ -9819,10 +9817,10 @@
       <c r="H4" t="inlineStr"/>
       <c r="I4" t="inlineStr"/>
       <c r="J4" t="inlineStr"/>
-      <c r="K4" t="inlineStr"/>
-      <c r="L4" t="n">
-        <v>1</v>
-      </c>
+      <c r="K4" t="n">
+        <v>1</v>
+      </c>
+      <c r="L4" t="inlineStr"/>
       <c r="M4" t="inlineStr"/>
       <c r="N4" t="inlineStr"/>
       <c r="O4" t="inlineStr"/>
@@ -9845,7 +9843,9 @@
       <c r="AB4" t="inlineStr"/>
       <c r="AC4" t="inlineStr"/>
       <c r="AD4" t="inlineStr"/>
-      <c r="AE4" t="inlineStr"/>
+      <c r="AE4" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -9911,16 +9911,16 @@
       <c r="L6" t="inlineStr"/>
       <c r="M6" t="inlineStr"/>
       <c r="N6" t="inlineStr"/>
-      <c r="O6" t="inlineStr"/>
+      <c r="O6" t="n">
+        <v>1</v>
+      </c>
       <c r="P6" t="inlineStr"/>
-      <c r="Q6" t="n">
-        <v>1</v>
-      </c>
+      <c r="Q6" t="inlineStr"/>
       <c r="R6" t="inlineStr"/>
-      <c r="S6" t="n">
-        <v>1</v>
-      </c>
-      <c r="T6" t="inlineStr"/>
+      <c r="S6" t="inlineStr"/>
+      <c r="T6" t="n">
+        <v>1</v>
+      </c>
       <c r="U6" t="inlineStr"/>
       <c r="V6" t="inlineStr"/>
       <c r="W6" t="inlineStr"/>
@@ -10058,10 +10058,10 @@
       <c r="A10" t="n">
         <v>9</v>
       </c>
-      <c r="B10" t="n">
-        <v>1</v>
-      </c>
-      <c r="C10" t="inlineStr"/>
+      <c r="B10" t="inlineStr"/>
+      <c r="C10" t="n">
+        <v>1</v>
+      </c>
       <c r="D10" t="inlineStr"/>
       <c r="E10" t="inlineStr"/>
       <c r="F10" t="inlineStr"/>
@@ -10069,30 +10069,30 @@
       <c r="H10" t="inlineStr"/>
       <c r="I10" t="inlineStr"/>
       <c r="J10" t="inlineStr"/>
-      <c r="K10" t="inlineStr"/>
-      <c r="L10" t="n">
-        <v>1</v>
-      </c>
+      <c r="K10" t="n">
+        <v>1</v>
+      </c>
+      <c r="L10" t="inlineStr"/>
       <c r="M10" t="inlineStr"/>
       <c r="N10" t="inlineStr"/>
       <c r="O10" t="inlineStr"/>
       <c r="P10" t="inlineStr"/>
-      <c r="Q10" t="inlineStr"/>
+      <c r="Q10" t="n">
+        <v>1</v>
+      </c>
       <c r="R10" t="inlineStr"/>
       <c r="S10" t="n">
         <v>1</v>
       </c>
-      <c r="T10" t="n">
-        <v>1</v>
-      </c>
+      <c r="T10" t="inlineStr"/>
       <c r="U10" t="inlineStr"/>
       <c r="V10" t="inlineStr"/>
       <c r="W10" t="inlineStr"/>
       <c r="X10" t="inlineStr"/>
-      <c r="Y10" t="n">
-        <v>1</v>
-      </c>
-      <c r="Z10" t="inlineStr"/>
+      <c r="Y10" t="inlineStr"/>
+      <c r="Z10" t="n">
+        <v>1</v>
+      </c>
       <c r="AA10" t="inlineStr"/>
       <c r="AB10" t="inlineStr"/>
       <c r="AC10" t="inlineStr"/>
@@ -10113,16 +10113,18 @@
       <c r="G11" t="inlineStr"/>
       <c r="H11" t="inlineStr"/>
       <c r="I11" t="inlineStr"/>
-      <c r="J11" t="inlineStr"/>
+      <c r="J11" t="n">
+        <v>1</v>
+      </c>
       <c r="K11" t="inlineStr"/>
-      <c r="L11" t="n">
-        <v>1</v>
-      </c>
+      <c r="L11" t="inlineStr"/>
       <c r="M11" t="inlineStr"/>
       <c r="N11" t="inlineStr"/>
       <c r="O11" t="inlineStr"/>
       <c r="P11" t="inlineStr"/>
-      <c r="Q11" t="inlineStr"/>
+      <c r="Q11" t="n">
+        <v>1</v>
+      </c>
       <c r="R11" t="n">
         <v>1</v>
       </c>
@@ -10130,21 +10132,17 @@
       <c r="T11" t="inlineStr"/>
       <c r="U11" t="inlineStr"/>
       <c r="V11" t="inlineStr"/>
-      <c r="W11" t="n">
-        <v>1</v>
-      </c>
+      <c r="W11" t="inlineStr"/>
       <c r="X11" t="inlineStr"/>
       <c r="Y11" t="inlineStr"/>
-      <c r="Z11" t="n">
-        <v>1</v>
-      </c>
+      <c r="Z11" t="inlineStr"/>
       <c r="AA11" t="inlineStr"/>
       <c r="AB11" t="inlineStr"/>
       <c r="AC11" t="inlineStr"/>
-      <c r="AD11" t="inlineStr"/>
-      <c r="AE11" t="n">
-        <v>1</v>
-      </c>
+      <c r="AD11" t="n">
+        <v>1</v>
+      </c>
+      <c r="AE11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="n">
@@ -10173,13 +10171,13 @@
       <c r="V12" t="inlineStr"/>
       <c r="W12" t="inlineStr"/>
       <c r="X12" t="inlineStr"/>
-      <c r="Y12" t="inlineStr"/>
+      <c r="Y12" t="n">
+        <v>1</v>
+      </c>
       <c r="Z12" t="n">
         <v>1</v>
       </c>
-      <c r="AA12" t="n">
-        <v>1</v>
-      </c>
+      <c r="AA12" t="inlineStr"/>
       <c r="AB12" t="inlineStr"/>
       <c r="AC12" t="inlineStr"/>
       <c r="AD12" t="inlineStr"/>
@@ -10194,9 +10192,7 @@
       <c r="B13" t="n">
         <v>1</v>
       </c>
-      <c r="C13" t="n">
-        <v>1</v>
-      </c>
+      <c r="C13" t="inlineStr"/>
       <c r="D13" t="inlineStr"/>
       <c r="E13" t="inlineStr"/>
       <c r="F13" t="inlineStr"/>
@@ -10207,24 +10203,26 @@
         <v>1</v>
       </c>
       <c r="K13" t="inlineStr"/>
-      <c r="L13" t="n">
-        <v>1</v>
-      </c>
+      <c r="L13" t="inlineStr"/>
       <c r="M13" t="inlineStr"/>
       <c r="N13" t="inlineStr"/>
       <c r="O13" t="inlineStr"/>
       <c r="P13" t="inlineStr"/>
-      <c r="Q13" t="inlineStr"/>
+      <c r="Q13" t="n">
+        <v>1</v>
+      </c>
       <c r="R13" t="inlineStr"/>
       <c r="S13" t="inlineStr"/>
-      <c r="T13" t="inlineStr"/>
+      <c r="T13" t="n">
+        <v>1</v>
+      </c>
       <c r="U13" t="inlineStr"/>
       <c r="V13" t="inlineStr"/>
-      <c r="W13" t="n">
-        <v>1</v>
-      </c>
+      <c r="W13" t="inlineStr"/>
       <c r="X13" t="inlineStr"/>
-      <c r="Y13" t="inlineStr"/>
+      <c r="Y13" t="n">
+        <v>1</v>
+      </c>
       <c r="Z13" t="n">
         <v>1</v>
       </c>
@@ -10241,9 +10239,7 @@
       <c r="B14" t="n">
         <v>1</v>
       </c>
-      <c r="C14" t="n">
-        <v>1</v>
-      </c>
+      <c r="C14" t="inlineStr"/>
       <c r="D14" t="inlineStr"/>
       <c r="E14" t="inlineStr"/>
       <c r="F14" t="inlineStr"/>
@@ -10253,25 +10249,27 @@
       <c r="J14" t="n">
         <v>1</v>
       </c>
-      <c r="K14" t="inlineStr"/>
+      <c r="K14" t="n">
+        <v>1</v>
+      </c>
       <c r="L14" t="inlineStr"/>
       <c r="M14" t="inlineStr"/>
       <c r="N14" t="inlineStr"/>
       <c r="O14" t="inlineStr"/>
-      <c r="P14" t="n">
-        <v>1</v>
-      </c>
-      <c r="Q14" t="inlineStr"/>
+      <c r="P14" t="inlineStr"/>
+      <c r="Q14" t="n">
+        <v>1</v>
+      </c>
       <c r="R14" t="inlineStr"/>
       <c r="S14" t="inlineStr"/>
-      <c r="T14" t="n">
-        <v>1</v>
-      </c>
+      <c r="T14" t="inlineStr"/>
       <c r="U14" t="inlineStr"/>
       <c r="V14" t="inlineStr"/>
       <c r="W14" t="inlineStr"/>
       <c r="X14" t="inlineStr"/>
-      <c r="Y14" t="inlineStr"/>
+      <c r="Y14" t="n">
+        <v>1</v>
+      </c>
       <c r="Z14" t="n">
         <v>1</v>
       </c>
@@ -10304,24 +10302,24 @@
       <c r="P15" t="inlineStr"/>
       <c r="Q15" t="inlineStr"/>
       <c r="R15" t="inlineStr"/>
-      <c r="S15" t="n">
-        <v>1</v>
-      </c>
-      <c r="T15" t="inlineStr"/>
+      <c r="S15" t="inlineStr"/>
+      <c r="T15" t="n">
+        <v>1</v>
+      </c>
       <c r="U15" t="inlineStr"/>
       <c r="V15" t="inlineStr"/>
       <c r="W15" t="inlineStr"/>
       <c r="X15" t="inlineStr"/>
-      <c r="Y15" t="inlineStr"/>
+      <c r="Y15" t="n">
+        <v>1</v>
+      </c>
       <c r="Z15" t="inlineStr"/>
       <c r="AA15" t="n">
         <v>1</v>
       </c>
       <c r="AB15" t="inlineStr"/>
       <c r="AC15" t="inlineStr"/>
-      <c r="AD15" t="n">
-        <v>1</v>
-      </c>
+      <c r="AD15" t="inlineStr"/>
       <c r="AE15" t="inlineStr"/>
     </row>
     <row r="16">
@@ -10341,10 +10339,10 @@
       <c r="H16" t="inlineStr"/>
       <c r="I16" t="inlineStr"/>
       <c r="J16" t="inlineStr"/>
-      <c r="K16" t="n">
-        <v>1</v>
-      </c>
-      <c r="L16" t="inlineStr"/>
+      <c r="K16" t="inlineStr"/>
+      <c r="L16" t="n">
+        <v>1</v>
+      </c>
       <c r="M16" t="inlineStr"/>
       <c r="N16" t="inlineStr"/>
       <c r="O16" t="inlineStr"/>
@@ -10366,10 +10364,10 @@
       <c r="AA16" t="inlineStr"/>
       <c r="AB16" t="inlineStr"/>
       <c r="AC16" t="inlineStr"/>
-      <c r="AD16" t="inlineStr"/>
-      <c r="AE16" t="n">
-        <v>1</v>
-      </c>
+      <c r="AD16" t="n">
+        <v>1</v>
+      </c>
+      <c r="AE16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="n">
@@ -10390,13 +10388,13 @@
       <c r="L17" t="inlineStr"/>
       <c r="M17" t="inlineStr"/>
       <c r="N17" t="inlineStr"/>
-      <c r="O17" t="n">
-        <v>1</v>
-      </c>
+      <c r="O17" t="inlineStr"/>
       <c r="P17" t="inlineStr"/>
       <c r="Q17" t="inlineStr"/>
       <c r="R17" t="inlineStr"/>
-      <c r="S17" t="inlineStr"/>
+      <c r="S17" t="n">
+        <v>1</v>
+      </c>
       <c r="T17" t="n">
         <v>1</v>
       </c>
@@ -10404,15 +10402,15 @@
       <c r="V17" t="inlineStr"/>
       <c r="W17" t="inlineStr"/>
       <c r="X17" t="inlineStr"/>
-      <c r="Y17" t="n">
-        <v>1</v>
-      </c>
+      <c r="Y17" t="inlineStr"/>
       <c r="Z17" t="inlineStr"/>
       <c r="AA17" t="inlineStr"/>
       <c r="AB17" t="inlineStr"/>
       <c r="AC17" t="inlineStr"/>
       <c r="AD17" t="inlineStr"/>
-      <c r="AE17" t="inlineStr"/>
+      <c r="AE17" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="n">
@@ -10428,18 +10426,18 @@
       <c r="G18" t="inlineStr"/>
       <c r="H18" t="inlineStr"/>
       <c r="I18" t="inlineStr"/>
-      <c r="J18" t="inlineStr"/>
+      <c r="J18" t="n">
+        <v>1</v>
+      </c>
       <c r="K18" t="inlineStr"/>
-      <c r="L18" t="inlineStr"/>
-      <c r="M18" t="n">
-        <v>1</v>
-      </c>
+      <c r="L18" t="n">
+        <v>1</v>
+      </c>
+      <c r="M18" t="inlineStr"/>
       <c r="N18" t="inlineStr"/>
       <c r="O18" t="inlineStr"/>
       <c r="P18" t="inlineStr"/>
-      <c r="Q18" t="n">
-        <v>1</v>
-      </c>
+      <c r="Q18" t="inlineStr"/>
       <c r="R18" t="n">
         <v>1</v>
       </c>
@@ -10450,7 +10448,9 @@
       <c r="W18" t="inlineStr"/>
       <c r="X18" t="inlineStr"/>
       <c r="Y18" t="inlineStr"/>
-      <c r="Z18" t="inlineStr"/>
+      <c r="Z18" t="n">
+        <v>1</v>
+      </c>
       <c r="AA18" t="inlineStr"/>
       <c r="AB18" t="inlineStr"/>
       <c r="AC18" t="inlineStr"/>
@@ -10490,13 +10490,13 @@
         <v>1</v>
       </c>
       <c r="Z19" t="inlineStr"/>
-      <c r="AA19" t="n">
-        <v>1</v>
-      </c>
+      <c r="AA19" t="inlineStr"/>
       <c r="AB19" t="inlineStr"/>
       <c r="AC19" t="inlineStr"/>
       <c r="AD19" t="inlineStr"/>
-      <c r="AE19" t="inlineStr"/>
+      <c r="AE19" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="n">
@@ -10512,16 +10512,18 @@
       <c r="G20" t="inlineStr"/>
       <c r="H20" t="inlineStr"/>
       <c r="I20" t="inlineStr"/>
-      <c r="J20" t="inlineStr"/>
+      <c r="J20" t="n">
+        <v>1</v>
+      </c>
       <c r="K20" t="inlineStr"/>
-      <c r="L20" t="inlineStr"/>
+      <c r="L20" t="n">
+        <v>1</v>
+      </c>
       <c r="M20" t="inlineStr"/>
       <c r="N20" t="inlineStr"/>
       <c r="O20" t="inlineStr"/>
       <c r="P20" t="inlineStr"/>
-      <c r="Q20" t="n">
-        <v>1</v>
-      </c>
+      <c r="Q20" t="inlineStr"/>
       <c r="R20" t="n">
         <v>1</v>
       </c>
@@ -10548,7 +10550,9 @@
         <v>20</v>
       </c>
       <c r="B21" t="inlineStr"/>
-      <c r="C21" t="inlineStr"/>
+      <c r="C21" t="n">
+        <v>1</v>
+      </c>
       <c r="D21" t="inlineStr"/>
       <c r="E21" t="inlineStr"/>
       <c r="F21" t="inlineStr"/>
@@ -10559,10 +10563,10 @@
       <c r="K21" t="n">
         <v>1</v>
       </c>
-      <c r="L21" t="inlineStr"/>
-      <c r="M21" t="n">
-        <v>1</v>
-      </c>
+      <c r="L21" t="n">
+        <v>1</v>
+      </c>
+      <c r="M21" t="inlineStr"/>
       <c r="N21" t="inlineStr"/>
       <c r="O21" t="inlineStr"/>
       <c r="P21" t="inlineStr"/>
@@ -10576,17 +10580,15 @@
       <c r="V21" t="inlineStr"/>
       <c r="W21" t="inlineStr"/>
       <c r="X21" t="inlineStr"/>
-      <c r="Y21" t="inlineStr"/>
-      <c r="Z21" t="n">
-        <v>1</v>
-      </c>
+      <c r="Y21" t="n">
+        <v>1</v>
+      </c>
+      <c r="Z21" t="inlineStr"/>
       <c r="AA21" t="inlineStr"/>
       <c r="AB21" t="inlineStr"/>
       <c r="AC21" t="inlineStr"/>
       <c r="AD21" t="inlineStr"/>
-      <c r="AE21" t="n">
-        <v>1</v>
-      </c>
+      <c r="AE21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="n">
@@ -10639,13 +10641,9 @@
       <c r="G23" t="inlineStr"/>
       <c r="H23" t="inlineStr"/>
       <c r="I23" t="inlineStr"/>
-      <c r="J23" t="n">
-        <v>1</v>
-      </c>
+      <c r="J23" t="inlineStr"/>
       <c r="K23" t="inlineStr"/>
-      <c r="L23" t="n">
-        <v>1</v>
-      </c>
+      <c r="L23" t="inlineStr"/>
       <c r="M23" t="inlineStr"/>
       <c r="N23" t="inlineStr"/>
       <c r="O23" t="inlineStr"/>
@@ -10668,7 +10666,9 @@
       <c r="AB23" t="inlineStr"/>
       <c r="AC23" t="inlineStr"/>
       <c r="AD23" t="inlineStr"/>
-      <c r="AE23" t="inlineStr"/>
+      <c r="AE23" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="n">
@@ -10685,13 +10685,11 @@
       <c r="H24" t="inlineStr"/>
       <c r="I24" t="inlineStr"/>
       <c r="J24" t="inlineStr"/>
-      <c r="K24" t="n">
-        <v>1</v>
-      </c>
-      <c r="L24" t="n">
-        <v>1</v>
-      </c>
-      <c r="M24" t="inlineStr"/>
+      <c r="K24" t="inlineStr"/>
+      <c r="L24" t="inlineStr"/>
+      <c r="M24" t="n">
+        <v>1</v>
+      </c>
       <c r="N24" t="inlineStr"/>
       <c r="O24" t="inlineStr"/>
       <c r="P24" t="inlineStr"/>
@@ -10700,15 +10698,17 @@
         <v>1</v>
       </c>
       <c r="S24" t="inlineStr"/>
-      <c r="T24" t="inlineStr"/>
+      <c r="T24" t="n">
+        <v>1</v>
+      </c>
       <c r="U24" t="inlineStr"/>
       <c r="V24" t="inlineStr"/>
       <c r="W24" t="inlineStr"/>
       <c r="X24" t="inlineStr"/>
-      <c r="Y24" t="n">
-        <v>1</v>
-      </c>
-      <c r="Z24" t="inlineStr"/>
+      <c r="Y24" t="inlineStr"/>
+      <c r="Z24" t="n">
+        <v>1</v>
+      </c>
       <c r="AA24" t="inlineStr"/>
       <c r="AB24" t="inlineStr"/>
       <c r="AC24" t="inlineStr"/>
@@ -10728,9 +10728,7 @@
       <c r="F25" t="inlineStr"/>
       <c r="G25" t="inlineStr"/>
       <c r="H25" t="inlineStr"/>
-      <c r="I25" t="n">
-        <v>1</v>
-      </c>
+      <c r="I25" t="inlineStr"/>
       <c r="J25" t="inlineStr"/>
       <c r="K25" t="inlineStr"/>
       <c r="L25" t="inlineStr"/>
@@ -10746,7 +10744,9 @@
       <c r="V25" t="inlineStr"/>
       <c r="W25" t="inlineStr"/>
       <c r="X25" t="inlineStr"/>
-      <c r="Y25" t="inlineStr"/>
+      <c r="Y25" t="n">
+        <v>1</v>
+      </c>
       <c r="Z25" t="inlineStr"/>
       <c r="AA25" t="n">
         <v>1</v>
@@ -10806,7 +10806,9 @@
       <c r="H27" t="inlineStr"/>
       <c r="I27" t="inlineStr"/>
       <c r="J27" t="inlineStr"/>
-      <c r="K27" t="inlineStr"/>
+      <c r="K27" t="n">
+        <v>1</v>
+      </c>
       <c r="L27" t="n">
         <v>1</v>
       </c>
@@ -10819,9 +10821,7 @@
         <v>1</v>
       </c>
       <c r="S27" t="inlineStr"/>
-      <c r="T27" t="n">
-        <v>1</v>
-      </c>
+      <c r="T27" t="inlineStr"/>
       <c r="U27" t="inlineStr"/>
       <c r="V27" t="inlineStr"/>
       <c r="W27" t="inlineStr"/>
@@ -10834,7 +10834,9 @@
       <c r="AB27" t="inlineStr"/>
       <c r="AC27" t="inlineStr"/>
       <c r="AD27" t="inlineStr"/>
-      <c r="AE27" t="inlineStr"/>
+      <c r="AE27" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="n">
@@ -10848,11 +10850,11 @@
       <c r="G28" t="inlineStr"/>
       <c r="H28" t="inlineStr"/>
       <c r="I28" t="inlineStr"/>
-      <c r="J28" t="n">
-        <v>1</v>
-      </c>
+      <c r="J28" t="inlineStr"/>
       <c r="K28" t="inlineStr"/>
-      <c r="L28" t="inlineStr"/>
+      <c r="L28" t="n">
+        <v>1</v>
+      </c>
       <c r="M28" t="inlineStr"/>
       <c r="N28" t="inlineStr"/>
       <c r="O28" t="inlineStr"/>
@@ -10869,11 +10871,11 @@
       <c r="V28" t="inlineStr"/>
       <c r="W28" t="inlineStr"/>
       <c r="X28" t="inlineStr"/>
-      <c r="Y28" t="n">
-        <v>1</v>
-      </c>
+      <c r="Y28" t="inlineStr"/>
       <c r="Z28" t="inlineStr"/>
-      <c r="AA28" t="inlineStr"/>
+      <c r="AA28" t="n">
+        <v>1</v>
+      </c>
       <c r="AB28" t="inlineStr"/>
       <c r="AC28" t="inlineStr"/>
       <c r="AD28" t="inlineStr"/>
@@ -10892,10 +10894,10 @@
       <c r="H29" t="inlineStr"/>
       <c r="I29" t="inlineStr"/>
       <c r="J29" t="inlineStr"/>
-      <c r="K29" t="n">
-        <v>1</v>
-      </c>
-      <c r="L29" t="inlineStr"/>
+      <c r="K29" t="inlineStr"/>
+      <c r="L29" t="n">
+        <v>1</v>
+      </c>
       <c r="M29" t="inlineStr"/>
       <c r="N29" t="inlineStr"/>
       <c r="O29" t="inlineStr"/>
@@ -10912,11 +10914,11 @@
       <c r="V29" t="inlineStr"/>
       <c r="W29" t="inlineStr"/>
       <c r="X29" t="inlineStr"/>
-      <c r="Y29" t="n">
-        <v>1</v>
-      </c>
+      <c r="Y29" t="inlineStr"/>
       <c r="Z29" t="inlineStr"/>
-      <c r="AA29" t="inlineStr"/>
+      <c r="AA29" t="n">
+        <v>1</v>
+      </c>
       <c r="AB29" t="inlineStr"/>
       <c r="AC29" t="inlineStr"/>
       <c r="AD29" t="inlineStr"/>
@@ -10935,22 +10937,22 @@
       <c r="H30" t="inlineStr"/>
       <c r="I30" t="inlineStr"/>
       <c r="J30" t="inlineStr"/>
-      <c r="K30" t="n">
-        <v>1</v>
-      </c>
+      <c r="K30" t="inlineStr"/>
       <c r="L30" t="inlineStr"/>
-      <c r="M30" t="inlineStr"/>
+      <c r="M30" t="n">
+        <v>1</v>
+      </c>
       <c r="N30" t="inlineStr"/>
       <c r="O30" t="inlineStr"/>
       <c r="P30" t="inlineStr"/>
-      <c r="Q30" t="n">
-        <v>1</v>
-      </c>
+      <c r="Q30" t="inlineStr"/>
       <c r="R30" t="inlineStr"/>
       <c r="S30" t="n">
         <v>1</v>
       </c>
-      <c r="T30" t="inlineStr"/>
+      <c r="T30" t="n">
+        <v>1</v>
+      </c>
       <c r="U30" t="inlineStr"/>
       <c r="V30" t="inlineStr"/>
       <c r="W30" t="inlineStr"/>
@@ -10982,9 +10984,7 @@
       <c r="H31" t="inlineStr"/>
       <c r="I31" t="inlineStr"/>
       <c r="J31" t="inlineStr"/>
-      <c r="K31" t="n">
-        <v>1</v>
-      </c>
+      <c r="K31" t="inlineStr"/>
       <c r="L31" t="n">
         <v>1</v>
       </c>
@@ -11004,7 +11004,9 @@
         <v>1</v>
       </c>
       <c r="X31" t="inlineStr"/>
-      <c r="Y31" t="inlineStr"/>
+      <c r="Y31" t="n">
+        <v>1</v>
+      </c>
       <c r="Z31" t="inlineStr"/>
       <c r="AA31" t="inlineStr"/>
       <c r="AB31" t="inlineStr"/>
@@ -11016,7 +11018,9 @@
       <c r="A32" t="n">
         <v>31</v>
       </c>
-      <c r="B32" t="inlineStr"/>
+      <c r="B32" t="n">
+        <v>1</v>
+      </c>
       <c r="C32" t="inlineStr"/>
       <c r="D32" t="inlineStr"/>
       <c r="E32" t="n">
@@ -11025,12 +11029,14 @@
       <c r="F32" t="inlineStr"/>
       <c r="G32" t="inlineStr"/>
       <c r="H32" t="inlineStr"/>
-      <c r="I32" t="inlineStr"/>
-      <c r="J32" t="n">
-        <v>1</v>
-      </c>
+      <c r="I32" t="n">
+        <v>1</v>
+      </c>
+      <c r="J32" t="inlineStr"/>
       <c r="K32" t="inlineStr"/>
-      <c r="L32" t="inlineStr"/>
+      <c r="L32" t="n">
+        <v>1</v>
+      </c>
       <c r="M32" t="inlineStr"/>
       <c r="N32" t="inlineStr"/>
       <c r="O32" t="inlineStr"/>
@@ -11040,9 +11046,7 @@
       </c>
       <c r="R32" t="inlineStr"/>
       <c r="S32" t="inlineStr"/>
-      <c r="T32" t="n">
-        <v>1</v>
-      </c>
+      <c r="T32" t="inlineStr"/>
       <c r="U32" t="inlineStr"/>
       <c r="V32" t="inlineStr"/>
       <c r="W32" t="inlineStr"/>
@@ -11055,15 +11059,15 @@
       <c r="AB32" t="inlineStr"/>
       <c r="AC32" t="inlineStr"/>
       <c r="AD32" t="inlineStr"/>
-      <c r="AE32" t="n">
-        <v>1</v>
-      </c>
+      <c r="AE32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="n">
         <v>32</v>
       </c>
-      <c r="B33" t="inlineStr"/>
+      <c r="B33" t="n">
+        <v>1</v>
+      </c>
       <c r="C33" t="inlineStr"/>
       <c r="D33" t="inlineStr"/>
       <c r="E33" t="n">
@@ -11077,19 +11081,17 @@
       <c r="K33" t="n">
         <v>1</v>
       </c>
-      <c r="L33" t="n">
-        <v>1</v>
-      </c>
+      <c r="L33" t="inlineStr"/>
       <c r="M33" t="inlineStr"/>
       <c r="N33" t="inlineStr"/>
       <c r="O33" t="inlineStr"/>
-      <c r="P33" t="inlineStr"/>
+      <c r="P33" t="n">
+        <v>1</v>
+      </c>
       <c r="Q33" t="inlineStr"/>
       <c r="R33" t="inlineStr"/>
       <c r="S33" t="inlineStr"/>
-      <c r="T33" t="n">
-        <v>1</v>
-      </c>
+      <c r="T33" t="inlineStr"/>
       <c r="U33" t="inlineStr"/>
       <c r="V33" t="inlineStr"/>
       <c r="W33" t="inlineStr"/>
@@ -11102,9 +11104,7 @@
       <c r="AB33" t="inlineStr"/>
       <c r="AC33" t="inlineStr"/>
       <c r="AD33" t="inlineStr"/>
-      <c r="AE33" t="n">
-        <v>1</v>
-      </c>
+      <c r="AE33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="n">
@@ -11121,9 +11121,7 @@
       <c r="H34" t="inlineStr"/>
       <c r="I34" t="inlineStr"/>
       <c r="J34" t="inlineStr"/>
-      <c r="K34" t="n">
-        <v>1</v>
-      </c>
+      <c r="K34" t="inlineStr"/>
       <c r="L34" t="n">
         <v>1</v>
       </c>
@@ -11141,11 +11139,13 @@
       <c r="V34" t="inlineStr"/>
       <c r="W34" t="inlineStr"/>
       <c r="X34" t="inlineStr"/>
-      <c r="Y34" t="inlineStr"/>
-      <c r="Z34" t="n">
-        <v>1</v>
-      </c>
-      <c r="AA34" t="inlineStr"/>
+      <c r="Y34" t="n">
+        <v>1</v>
+      </c>
+      <c r="Z34" t="inlineStr"/>
+      <c r="AA34" t="n">
+        <v>1</v>
+      </c>
       <c r="AB34" t="inlineStr"/>
       <c r="AC34" t="inlineStr"/>
       <c r="AD34" t="inlineStr"/>
@@ -11214,7 +11214,9 @@
       <c r="M36" t="inlineStr"/>
       <c r="N36" t="inlineStr"/>
       <c r="O36" t="inlineStr"/>
-      <c r="P36" t="inlineStr"/>
+      <c r="P36" t="n">
+        <v>1</v>
+      </c>
       <c r="Q36" t="inlineStr"/>
       <c r="R36" t="inlineStr"/>
       <c r="S36" t="inlineStr"/>
@@ -11230,9 +11232,7 @@
       <c r="AA36" t="inlineStr"/>
       <c r="AB36" t="inlineStr"/>
       <c r="AC36" t="inlineStr"/>
-      <c r="AD36" t="n">
-        <v>1</v>
-      </c>
+      <c r="AD36" t="inlineStr"/>
       <c r="AE36" t="inlineStr"/>
     </row>
     <row r="37">
@@ -11249,28 +11249,30 @@
       <c r="G37" t="inlineStr"/>
       <c r="H37" t="inlineStr"/>
       <c r="I37" t="inlineStr"/>
-      <c r="J37" t="inlineStr"/>
-      <c r="K37" t="inlineStr"/>
-      <c r="L37" t="n">
-        <v>1</v>
-      </c>
+      <c r="J37" t="n">
+        <v>1</v>
+      </c>
+      <c r="K37" t="n">
+        <v>1</v>
+      </c>
+      <c r="L37" t="inlineStr"/>
       <c r="M37" t="inlineStr"/>
       <c r="N37" t="inlineStr"/>
       <c r="O37" t="inlineStr"/>
-      <c r="P37" t="n">
-        <v>1</v>
-      </c>
-      <c r="Q37" t="inlineStr"/>
+      <c r="P37" t="inlineStr"/>
+      <c r="Q37" t="n">
+        <v>1</v>
+      </c>
       <c r="R37" t="inlineStr"/>
       <c r="S37" t="inlineStr"/>
-      <c r="T37" t="inlineStr"/>
+      <c r="T37" t="n">
+        <v>1</v>
+      </c>
       <c r="U37" t="inlineStr"/>
       <c r="V37" t="inlineStr"/>
       <c r="W37" t="inlineStr"/>
       <c r="X37" t="inlineStr"/>
-      <c r="Y37" t="n">
-        <v>1</v>
-      </c>
+      <c r="Y37" t="inlineStr"/>
       <c r="Z37" t="n">
         <v>1</v>
       </c>
@@ -11278,17 +11280,13 @@
       <c r="AB37" t="inlineStr"/>
       <c r="AC37" t="inlineStr"/>
       <c r="AD37" t="inlineStr"/>
-      <c r="AE37" t="n">
-        <v>1</v>
-      </c>
+      <c r="AE37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="n">
         <v>37</v>
       </c>
-      <c r="B38" t="n">
-        <v>1</v>
-      </c>
+      <c r="B38" t="inlineStr"/>
       <c r="C38" t="n">
         <v>1</v>
       </c>
@@ -11315,17 +11313,19 @@
       <c r="T38" t="inlineStr"/>
       <c r="U38" t="inlineStr"/>
       <c r="V38" t="inlineStr"/>
-      <c r="W38" t="inlineStr"/>
+      <c r="W38" t="n">
+        <v>1</v>
+      </c>
       <c r="X38" t="inlineStr"/>
-      <c r="Y38" t="n">
-        <v>1</v>
-      </c>
+      <c r="Y38" t="inlineStr"/>
       <c r="Z38" t="inlineStr"/>
       <c r="AA38" t="inlineStr"/>
       <c r="AB38" t="inlineStr"/>
       <c r="AC38" t="inlineStr"/>
       <c r="AD38" t="inlineStr"/>
-      <c r="AE38" t="inlineStr"/>
+      <c r="AE38" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="n">
@@ -11358,13 +11358,13 @@
       </c>
       <c r="U39" t="inlineStr"/>
       <c r="V39" t="inlineStr"/>
-      <c r="W39" t="inlineStr"/>
+      <c r="W39" t="n">
+        <v>1</v>
+      </c>
       <c r="X39" t="inlineStr"/>
       <c r="Y39" t="inlineStr"/>
       <c r="Z39" t="inlineStr"/>
-      <c r="AA39" t="n">
-        <v>1</v>
-      </c>
+      <c r="AA39" t="inlineStr"/>
       <c r="AB39" t="inlineStr"/>
       <c r="AC39" t="inlineStr"/>
       <c r="AD39" t="inlineStr"/>
@@ -11386,11 +11386,11 @@
       <c r="G40" t="inlineStr"/>
       <c r="H40" t="inlineStr"/>
       <c r="I40" t="inlineStr"/>
-      <c r="J40" t="inlineStr"/>
+      <c r="J40" t="n">
+        <v>1</v>
+      </c>
       <c r="K40" t="inlineStr"/>
-      <c r="L40" t="n">
-        <v>1</v>
-      </c>
+      <c r="L40" t="inlineStr"/>
       <c r="M40" t="inlineStr"/>
       <c r="N40" t="inlineStr"/>
       <c r="O40" t="inlineStr"/>
@@ -11410,10 +11410,10 @@
       <c r="W40" t="inlineStr"/>
       <c r="X40" t="inlineStr"/>
       <c r="Y40" t="inlineStr"/>
-      <c r="Z40" t="inlineStr"/>
-      <c r="AA40" t="n">
-        <v>1</v>
-      </c>
+      <c r="Z40" t="n">
+        <v>1</v>
+      </c>
+      <c r="AA40" t="inlineStr"/>
       <c r="AB40" t="inlineStr"/>
       <c r="AC40" t="inlineStr"/>
       <c r="AD40" t="inlineStr"/>
@@ -11450,11 +11450,13 @@
       <c r="V41" t="inlineStr"/>
       <c r="W41" t="inlineStr"/>
       <c r="X41" t="inlineStr"/>
-      <c r="Y41" t="inlineStr"/>
-      <c r="Z41" t="n">
-        <v>1</v>
-      </c>
-      <c r="AA41" t="inlineStr"/>
+      <c r="Y41" t="n">
+        <v>1</v>
+      </c>
+      <c r="Z41" t="inlineStr"/>
+      <c r="AA41" t="n">
+        <v>1</v>
+      </c>
       <c r="AB41" t="inlineStr"/>
       <c r="AC41" t="inlineStr"/>
       <c r="AD41" t="inlineStr"/>
@@ -11464,7 +11466,9 @@
       <c r="A42" t="n">
         <v>41</v>
       </c>
-      <c r="B42" t="inlineStr"/>
+      <c r="B42" t="n">
+        <v>1</v>
+      </c>
       <c r="C42" t="n">
         <v>1</v>
       </c>
@@ -11474,11 +11478,13 @@
       <c r="G42" t="inlineStr"/>
       <c r="H42" t="inlineStr"/>
       <c r="I42" t="inlineStr"/>
-      <c r="J42" t="n">
-        <v>1</v>
-      </c>
-      <c r="K42" t="inlineStr"/>
-      <c r="L42" t="inlineStr"/>
+      <c r="J42" t="inlineStr"/>
+      <c r="K42" t="n">
+        <v>1</v>
+      </c>
+      <c r="L42" t="n">
+        <v>1</v>
+      </c>
       <c r="M42" t="inlineStr"/>
       <c r="N42" t="inlineStr"/>
       <c r="O42" t="inlineStr"/>
@@ -11488,24 +11494,18 @@
       <c r="Q42" t="inlineStr"/>
       <c r="R42" t="inlineStr"/>
       <c r="S42" t="inlineStr"/>
-      <c r="T42" t="n">
-        <v>1</v>
-      </c>
+      <c r="T42" t="inlineStr"/>
       <c r="U42" t="inlineStr"/>
       <c r="V42" t="inlineStr"/>
       <c r="W42" t="inlineStr"/>
       <c r="X42" t="inlineStr"/>
-      <c r="Y42" t="n">
-        <v>1</v>
-      </c>
+      <c r="Y42" t="inlineStr"/>
       <c r="Z42" t="inlineStr"/>
       <c r="AA42" t="inlineStr"/>
       <c r="AB42" t="inlineStr"/>
       <c r="AC42" t="inlineStr"/>
       <c r="AD42" t="inlineStr"/>
-      <c r="AE42" t="n">
-        <v>1</v>
-      </c>
+      <c r="AE42" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>